<commit_message>
docs: refresh test case workbook with latest execution results
</commit_message>
<xml_diff>
--- a/test-cases/ParaBank_Test_Cases.xlsx
+++ b/test-cases/ParaBank_Test_Cases.xlsx
@@ -24,12 +24,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="353">
   <si>
     <t xml:space="preserve">ParaBank Sign-Up &amp; Login Automation  -  Test Case Suite</t>
   </si>
   <si>
-    <t xml:space="preserve">Application: https://parabank.parasoft.com/parabank/  |  Framework: Playwright + TypeScript  |  Style: BDD (Gherkin) + Page Object Model  |  33 test cases - all automated</t>
+    <t xml:space="preserve">Application: https://parabank.parasoft.com/parabank/   |   Framework: Playwright + TypeScript, BDD + POM   |   33 automated test cases   |   Latest run: 24-May-2026 - PASS (33 / 33)</t>
   </si>
   <si>
     <t xml:space="preserve">TC ID</t>
@@ -122,7 +122,7 @@
     <t xml:space="preserve">P1 - High</t>
   </si>
   <si>
-    <t xml:space="preserve">Not Run</t>
+    <t xml:space="preserve">Pass</t>
   </si>
   <si>
     <t xml:space="preserve">TC-002</t>
@@ -326,7 +326,7 @@
   </si>
   <si>
     <t xml:space="preserve">1. Open /register.htm.
-2. Fill each field with long (50-80 character) values.
+2. Fill each field with long (24-40 character) values.
 3. Click 'Register'.</t>
   </si>
   <si>
@@ -498,6 +498,9 @@
     <t xml:space="preserve">Expected: the injected markup is escaped and never rendered as live page content.</t>
   </si>
   <si>
+    <t xml:space="preserve">Observation</t>
+  </si>
+  <si>
     <t xml:space="preserve">KNOWN DEFECT: ParaBank renders the first name unescaped, confirming a stored XSS / HTML-injection exposure. The scenario is tagged @fail (expected failure) so the regression suite stays green while flagging the issue.</t>
   </si>
   <si>
@@ -824,6 +827,18 @@
     <t xml:space="preserve">5</t>
   </si>
   <si>
+    <t xml:space="preserve">Latest run date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24-May-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latest run result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASS - 33 / 33 checks passed</t>
+  </si>
+  <si>
     <t xml:space="preserve">Automation Mapping  -  BDD Scenario &lt;-&gt; Test Case</t>
   </si>
   <si>
@@ -971,13 +986,22 @@
     <t xml:space="preserve">% of Suite</t>
   </si>
   <si>
-    <t xml:space="preserve">Execution Status</t>
+    <t xml:space="preserve">Latest Execution  -  24-May-2026</t>
   </si>
   <si>
     <t xml:space="preserve">Note</t>
   </si>
   <si>
-    <t xml:space="preserve">Suite is ready to run. Execute 'npm test' locally and record Pass / Fail results.</t>
+    <t xml:space="preserve">Checks that passed cleanly in the automated run.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-019 - confirmed XSS exposure; runs as an expected failure (@fail) so the suite stays green.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASS  -  33 / 33 checks passed in 141 s.  The automated runner reports all 33 scenarios as passed.</t>
   </si>
   <si>
     <t xml:space="preserve">Documentation Guidelines &amp; Conventions</t>
@@ -1046,9 +1070,6 @@
     <t xml:space="preserve">Green</t>
   </si>
   <si>
-    <t xml:space="preserve">Pass</t>
-  </si>
-  <si>
     <t xml:space="preserve">Red</t>
   </si>
   <si>
@@ -1058,10 +1079,10 @@
     <t xml:space="preserve">Yellow</t>
   </si>
   <si>
+    <t xml:space="preserve">Not Run</t>
+  </si>
+  <si>
     <t xml:space="preserve">Blue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Observation</t>
   </si>
   <si>
     <t xml:space="preserve">Purple</t>
@@ -1125,7 +1146,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1205,7 +1226,15 @@
     <font>
       <b val="true"/>
       <sz val="8"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF1E7B34"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="8"/>
+      <color rgb="FF2F5496"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1266,14 +1295,6 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="8"/>
-      <color rgb="FF1E7B34"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
       <sz val="18"/>
       <color rgb="FF1F3864"/>
       <name val="Arial"/>
@@ -1289,16 +1310,24 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF9C6500"/>
+      <sz val="9"/>
+      <color rgb="FF595959"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF2F5496"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="9"/>
-      <color rgb="FF595959"/>
+      <color rgb="FF1E7B34"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1358,8 +1387,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFCE4D6"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -1370,8 +1399,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFCE4D6"/>
         <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBDD7EE"/>
+        <bgColor rgb="FFD9E2F3"/>
       </patternFill>
     </fill>
     <fill>
@@ -1394,12 +1435,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor rgb="FFE2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
         <bgColor rgb="FFEAD1DC"/>
       </patternFill>
@@ -1408,12 +1443,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
         <bgColor rgb="FFFFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFBDD7EE"/>
-        <bgColor rgb="FFD9E2F3"/>
       </patternFill>
     </fill>
     <fill>
@@ -1472,7 +1501,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="60">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1525,10 +1554,6 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1537,15 +1562,23 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1553,31 +1586,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1585,15 +1618,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1609,11 +1642,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1625,16 +1658,12 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1645,7 +1674,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1653,19 +1686,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1673,31 +1714,31 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="17" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="17" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1723,7 +1764,7 @@
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF1E7B34"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF9C6500"/>
+      <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
@@ -3028,16 +3069,16 @@
       <c r="N25" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="O25" s="9" t="s">
-        <v>31</v>
+      <c r="O25" s="15" t="s">
+        <v>143</v>
       </c>
       <c r="P25" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>20</v>
@@ -3055,25 +3096,25 @@
         <v>117</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I26" s="12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J26" s="12" t="s">
         <v>35</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L26" s="12" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M26" s="12" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N26" s="11" t="s">
         <v>39</v>
@@ -3085,7 +3126,7 @@
     </row>
     <row r="27" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>21</v>
@@ -3106,22 +3147,22 @@
         <v>48</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J27" s="8" t="s">
         <v>64</v>
       </c>
       <c r="K27" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="L27" s="8" t="s">
         <v>66</v>
       </c>
       <c r="M27" s="8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N27" s="6" t="s">
         <v>30</v>
@@ -3133,7 +3174,7 @@
     </row>
     <row r="28" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>21</v>
@@ -3154,22 +3195,22 @@
         <v>48</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I28" s="12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J28" s="12" t="s">
         <v>64</v>
       </c>
       <c r="K28" s="12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="L28" s="12" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="M28" s="12" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="N28" s="11" t="s">
         <v>39</v>
@@ -3181,7 +3222,7 @@
     </row>
     <row r="29" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>21</v>
@@ -3202,22 +3243,22 @@
         <v>48</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J29" s="8" t="s">
         <v>57</v>
       </c>
       <c r="K29" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L29" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="M29" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="N29" s="6" t="s">
         <v>39</v>
@@ -3229,7 +3270,7 @@
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -3249,7 +3290,7 @@
     </row>
     <row r="31" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>21</v>
@@ -3263,29 +3304,29 @@
       <c r="E31" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="F31" s="15" t="s">
-        <v>170</v>
+      <c r="F31" s="16" t="s">
+        <v>171</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H31" s="12" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I31" s="12" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J31" s="12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K31" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="L31" s="12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="M31" s="12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="N31" s="11" t="s">
         <v>30</v>
@@ -3297,7 +3338,7 @@
     </row>
     <row r="32" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>21</v>
@@ -3311,29 +3352,29 @@
       <c r="E32" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F32" s="15" t="s">
-        <v>170</v>
+      <c r="F32" s="16" t="s">
+        <v>171</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K32" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="L32" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="M32" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="N32" s="6" t="s">
         <v>39</v>
@@ -3345,7 +3386,7 @@
     </row>
     <row r="33" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>21</v>
@@ -3359,29 +3400,29 @@
       <c r="E33" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="F33" s="15" t="s">
-        <v>170</v>
+      <c r="F33" s="16" t="s">
+        <v>171</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I33" s="12" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J33" s="12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K33" s="12" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="L33" s="12" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="M33" s="12" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="N33" s="11" t="s">
         <v>39</v>
@@ -3393,7 +3434,7 @@
     </row>
     <row r="34" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>21</v>
@@ -3407,29 +3448,29 @@
       <c r="E34" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F34" s="15" t="s">
-        <v>170</v>
+      <c r="F34" s="16" t="s">
+        <v>171</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J34" s="8" t="s">
         <v>64</v>
       </c>
       <c r="K34" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L34" s="8" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="M34" s="8" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="N34" s="6" t="s">
         <v>30</v>
@@ -3441,7 +3482,7 @@
     </row>
     <row r="35" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>21</v>
@@ -3455,29 +3496,29 @@
       <c r="E35" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="F35" s="15" t="s">
-        <v>170</v>
+      <c r="F35" s="16" t="s">
+        <v>171</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H35" s="12" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I35" s="12" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J35" s="12" t="s">
         <v>64</v>
       </c>
       <c r="K35" s="12" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="L35" s="12" t="s">
         <v>66</v>
       </c>
       <c r="M35" s="12" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="N35" s="11" t="s">
         <v>39</v>
@@ -3489,7 +3530,7 @@
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -3509,7 +3550,7 @@
     </row>
     <row r="37" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>21</v>
@@ -3523,29 +3564,29 @@
       <c r="E37" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F37" s="16" t="s">
-        <v>201</v>
+      <c r="F37" s="17" t="s">
+        <v>202</v>
       </c>
       <c r="G37" s="8" t="s">
         <v>48</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J37" s="8" t="s">
         <v>35</v>
       </c>
       <c r="K37" s="8" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="L37" s="8" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="M37" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="N37" s="6" t="s">
         <v>89</v>
@@ -3557,7 +3598,7 @@
     </row>
     <row r="38" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>21</v>
@@ -3571,29 +3612,29 @@
       <c r="E38" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="F38" s="16" t="s">
-        <v>201</v>
+      <c r="F38" s="17" t="s">
+        <v>202</v>
       </c>
       <c r="G38" s="12" t="s">
         <v>23</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I38" s="12" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J38" s="12" t="s">
         <v>35</v>
       </c>
       <c r="K38" s="12" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="L38" s="12" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="M38" s="12" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="N38" s="11" t="s">
         <v>89</v>
@@ -3605,7 +3646,7 @@
     </row>
     <row r="39" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>21</v>
@@ -3619,29 +3660,29 @@
       <c r="E39" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F39" s="16" t="s">
-        <v>201</v>
+      <c r="F39" s="17" t="s">
+        <v>202</v>
       </c>
       <c r="G39" s="8" t="s">
         <v>23</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J39" s="8" t="s">
         <v>73</v>
       </c>
       <c r="K39" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="L39" s="8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="M39" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="N39" s="6" t="s">
         <v>89</v>
@@ -3653,7 +3694,7 @@
     </row>
     <row r="40" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>21</v>
@@ -3667,29 +3708,29 @@
       <c r="E40" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="F40" s="16" t="s">
-        <v>201</v>
+      <c r="F40" s="17" t="s">
+        <v>202</v>
       </c>
       <c r="G40" s="12" t="s">
         <v>48</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I40" s="12" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J40" s="12" t="s">
         <v>64</v>
       </c>
       <c r="K40" s="12" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="L40" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="M40" s="12" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="N40" s="11" t="s">
         <v>89</v>
@@ -3701,7 +3742,7 @@
     </row>
     <row r="41" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>21</v>
@@ -3715,29 +3756,29 @@
       <c r="E41" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F41" s="16" t="s">
-        <v>201</v>
+      <c r="F41" s="17" t="s">
+        <v>202</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J41" s="8" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K41" s="8" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="L41" s="8" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="M41" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="N41" s="6" t="s">
         <v>89</v>
@@ -3772,7 +3813,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -3780,295 +3821,311 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>225</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
+      <c r="A1" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
     </row>
     <row r="3" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
-        <v>226</v>
-      </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
+      <c r="A3" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="19" t="s">
-        <v>227</v>
-      </c>
-      <c r="C4" s="19" t="s">
+      <c r="B4" s="20" t="s">
         <v>228</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="C4" s="20" t="s">
         <v>229</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="D4" s="20" t="s">
         <v>230</v>
       </c>
+      <c r="E4" s="20" t="s">
+        <v>231</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Functional")</f>
         <v>6</v>
       </c>
-      <c r="C5" s="21" t="n">
+      <c r="C5" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Functional")</f>
         <v>6</v>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="22" t="s">
-        <v>231</v>
+      <c r="E5" s="23" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="21" t="n">
+      <c r="B6" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Boundary")</f>
         <v>8</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Boundary")</f>
         <v>8</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="D6" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="22" t="s">
-        <v>231</v>
+      <c r="E6" s="23" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="B7" s="21" t="n">
+      <c r="B7" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Security")</f>
         <v>9</v>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Security")</f>
         <v>9</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="22" t="s">
-        <v>231</v>
+      <c r="E7" s="23" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
-        <v>170</v>
-      </c>
-      <c r="B8" s="21" t="n">
+      <c r="A8" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="B8" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Access Control")</f>
         <v>5</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Access Control")</f>
         <v>5</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="22" t="s">
-        <v>231</v>
+      <c r="E8" s="23" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="26" t="s">
-        <v>201</v>
-      </c>
-      <c r="B9" s="21" t="n">
+      <c r="A9" s="27" t="s">
+        <v>202</v>
+      </c>
+      <c r="B9" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Performance")</f>
         <v>5</v>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Performance")</f>
         <v>5</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="22" t="s">
-        <v>231</v>
+      <c r="E9" s="23" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="27" t="s">
-        <v>232</v>
-      </c>
-      <c r="B10" s="28" t="n">
+      <c r="A10" s="28" t="s">
+        <v>233</v>
+      </c>
+      <c r="B10" s="29" t="n">
         <f aca="false">SUM(B5:B9)</f>
         <v>33</v>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="29" t="n">
         <f aca="false">SUM(C5:C9)</f>
         <v>33</v>
       </c>
-      <c r="D10" s="28" t="n">
+      <c r="D10" s="29" t="n">
         <f aca="false">SUM(D5:D9)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="29" t="s">
-        <v>231</v>
+      <c r="E10" s="30" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
+      <c r="A12" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="19" t="s">
-        <v>234</v>
-      </c>
-      <c r="C13" s="19" t="s">
+      <c r="B13" s="20" t="s">
         <v>235</v>
       </c>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
+      <c r="C13" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="21" t="n">
+      <c r="B14" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!N5:N41,"P1 - High")</f>
         <v>7</v>
       </c>
-      <c r="C14" s="21" t="str">
+      <c r="C14" s="22" t="str">
         <f aca="false">TEXT(B14/B10,"0%")</f>
         <v>21%</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="21" t="n">
+      <c r="B15" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!N5:N41,"P2 - Medium")</f>
         <v>18</v>
       </c>
-      <c r="C15" s="21" t="str">
+      <c r="C15" s="22" t="str">
         <f aca="false">TEXT(B15/B10,"0%")</f>
         <v>55%</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!N5:N41,"P3 - Low")</f>
         <v>8</v>
       </c>
-      <c r="C16" s="21" t="str">
+      <c r="C16" s="22" t="str">
         <f aca="false">TEXT(B16/B10,"0%")</f>
         <v>24%</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
-        <v>236</v>
-      </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="A18" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
-        <v>237</v>
-      </c>
-      <c r="B19" s="19" t="s">
+      <c r="A19" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
+      <c r="B19" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="30" t="s">
-        <v>239</v>
-      </c>
-      <c r="B20" s="21" t="n">
+      <c r="A20" s="31" t="s">
+        <v>240</v>
+      </c>
+      <c r="B20" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!A5:A41,"TC-*")</f>
         <v>33</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="30" t="s">
-        <v>240</v>
-      </c>
-      <c r="B21" s="21" t="n">
+      <c r="A21" s="31" t="s">
+        <v>241</v>
+      </c>
+      <c r="B21" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!A5:A41,"TC-*")</f>
         <v>33</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="30" t="s">
-        <v>241</v>
-      </c>
-      <c r="B22" s="21" t="n">
+      <c r="A22" s="31" t="s">
+        <v>242</v>
+      </c>
+      <c r="B22" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!B5:B41,"Y")</f>
         <v>4</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="30" t="s">
-        <v>242</v>
-      </c>
-      <c r="B23" s="21" t="n">
+      <c r="A23" s="31" t="s">
+        <v>243</v>
+      </c>
+      <c r="B23" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!D5:D41,"Y")</f>
         <v>9</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="30" t="s">
-        <v>243</v>
-      </c>
-      <c r="B24" s="21" t="n">
+      <c r="A24" s="31" t="s">
+        <v>244</v>
+      </c>
+      <c r="B24" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!A5:A41,"TC-*")</f>
         <v>33</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="30" t="s">
-        <v>244</v>
-      </c>
-      <c r="B25" s="21" t="s">
+      <c r="A25" s="31" t="s">
         <v>245</v>
       </c>
+      <c r="B25" s="22" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="30" t="s">
-        <v>246</v>
-      </c>
-      <c r="B26" s="21" t="s">
+      <c r="A26" s="31" t="s">
         <v>247</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="31" t="s">
+        <v>249</v>
+      </c>
+      <c r="B27" s="22" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="31" t="s">
+        <v>251</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -4105,18 +4162,18 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>248</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
+      <c r="A1" s="18" t="s">
+        <v>253</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4125,683 +4182,683 @@
       <c r="F2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="19" t="s">
-        <v>250</v>
-      </c>
-      <c r="D3" s="19" t="s">
-        <v>251</v>
-      </c>
-      <c r="E3" s="19" t="s">
-        <v>252</v>
-      </c>
-      <c r="F3" s="19" t="s">
-        <v>228</v>
+      <c r="C3" s="20" t="s">
+        <v>255</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>256</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>257</v>
+      </c>
+      <c r="F3" s="20" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="33" t="s">
-        <v>253</v>
-      </c>
-      <c r="D4" s="33" t="s">
+      <c r="C4" s="34" t="s">
+        <v>258</v>
+      </c>
+      <c r="D4" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="34" t="s">
-        <v>254</v>
-      </c>
-      <c r="F4" s="35" t="s">
-        <v>255</v>
+      <c r="E4" s="35" t="s">
+        <v>259</v>
+      </c>
+      <c r="F4" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="37" t="s">
-        <v>253</v>
-      </c>
-      <c r="D5" s="37" t="s">
+      <c r="C5" s="38" t="s">
+        <v>258</v>
+      </c>
+      <c r="D5" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="38" t="s">
-        <v>256</v>
-      </c>
-      <c r="F5" s="39" t="s">
-        <v>255</v>
+      <c r="E5" s="39" t="s">
+        <v>261</v>
+      </c>
+      <c r="F5" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="33" t="s">
-        <v>253</v>
-      </c>
-      <c r="D6" s="33" t="s">
+      <c r="C6" s="34" t="s">
+        <v>258</v>
+      </c>
+      <c r="D6" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="34" t="s">
-        <v>256</v>
-      </c>
-      <c r="F6" s="35" t="s">
-        <v>255</v>
+      <c r="E6" s="35" t="s">
+        <v>261</v>
+      </c>
+      <c r="F6" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="37" t="s">
-        <v>257</v>
-      </c>
-      <c r="D7" s="37" t="s">
-        <v>258</v>
-      </c>
-      <c r="E7" s="38" t="s">
-        <v>259</v>
-      </c>
-      <c r="F7" s="39" t="s">
-        <v>255</v>
+      <c r="C7" s="38" t="s">
+        <v>262</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>263</v>
+      </c>
+      <c r="E7" s="39" t="s">
+        <v>264</v>
+      </c>
+      <c r="F7" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="33" t="s">
-        <v>257</v>
-      </c>
-      <c r="D8" s="33" t="s">
+      <c r="C8" s="34" t="s">
+        <v>262</v>
+      </c>
+      <c r="D8" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="34" t="s">
+      <c r="E8" s="35" t="s">
+        <v>265</v>
+      </c>
+      <c r="F8" s="36" t="s">
         <v>260</v>
       </c>
-      <c r="F8" s="35" t="s">
-        <v>255</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="37" t="s">
-        <v>257</v>
-      </c>
-      <c r="D9" s="37" t="s">
+      <c r="C9" s="38" t="s">
+        <v>262</v>
+      </c>
+      <c r="D9" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="38" t="s">
-        <v>261</v>
-      </c>
-      <c r="F9" s="39" t="s">
-        <v>255</v>
+      <c r="E9" s="39" t="s">
+        <v>266</v>
+      </c>
+      <c r="F9" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="33" t="s">
-        <v>262</v>
-      </c>
-      <c r="D10" s="33" t="s">
+      <c r="C10" s="34" t="s">
+        <v>267</v>
+      </c>
+      <c r="D10" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="E10" s="34" t="s">
-        <v>263</v>
-      </c>
-      <c r="F10" s="35" t="s">
-        <v>255</v>
+      <c r="E10" s="35" t="s">
+        <v>268</v>
+      </c>
+      <c r="F10" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="36" t="s">
+      <c r="A11" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="37" t="s">
-        <v>262</v>
-      </c>
-      <c r="D11" s="37" t="s">
+      <c r="C11" s="38" t="s">
+        <v>267</v>
+      </c>
+      <c r="D11" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="E11" s="38" t="s">
-        <v>263</v>
-      </c>
-      <c r="F11" s="39" t="s">
-        <v>255</v>
+      <c r="E11" s="39" t="s">
+        <v>268</v>
+      </c>
+      <c r="F11" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="31" t="s">
+      <c r="A12" s="32" t="s">
         <v>83</v>
       </c>
-      <c r="B12" s="40" t="s">
+      <c r="B12" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="C12" s="33" t="s">
-        <v>262</v>
-      </c>
-      <c r="D12" s="33" t="s">
-        <v>264</v>
-      </c>
-      <c r="E12" s="34" t="s">
-        <v>265</v>
-      </c>
-      <c r="F12" s="35" t="s">
-        <v>255</v>
+      <c r="C12" s="34" t="s">
+        <v>267</v>
+      </c>
+      <c r="D12" s="34" t="s">
+        <v>269</v>
+      </c>
+      <c r="E12" s="35" t="s">
+        <v>270</v>
+      </c>
+      <c r="F12" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="36" t="s">
+      <c r="A13" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="37" t="s">
-        <v>262</v>
-      </c>
-      <c r="D13" s="37" t="s">
-        <v>266</v>
-      </c>
-      <c r="E13" s="38" t="s">
-        <v>265</v>
-      </c>
-      <c r="F13" s="39" t="s">
-        <v>255</v>
+      <c r="C13" s="38" t="s">
+        <v>267</v>
+      </c>
+      <c r="D13" s="38" t="s">
+        <v>271</v>
+      </c>
+      <c r="E13" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="F13" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="B14" s="40" t="s">
+      <c r="B14" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="C14" s="33" t="s">
-        <v>262</v>
-      </c>
-      <c r="D14" s="33" t="s">
+      <c r="C14" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="E14" s="34" t="s">
-        <v>265</v>
-      </c>
-      <c r="F14" s="35" t="s">
-        <v>255</v>
+      <c r="D14" s="34" t="s">
+        <v>272</v>
+      </c>
+      <c r="E14" s="35" t="s">
+        <v>270</v>
+      </c>
+      <c r="F14" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="36" t="s">
+      <c r="A15" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="C15" s="37" t="s">
-        <v>262</v>
-      </c>
-      <c r="D15" s="37" t="s">
+      <c r="C15" s="38" t="s">
+        <v>267</v>
+      </c>
+      <c r="D15" s="38" t="s">
+        <v>273</v>
+      </c>
+      <c r="E15" s="39" t="s">
         <v>268</v>
       </c>
-      <c r="E15" s="38" t="s">
-        <v>263</v>
-      </c>
-      <c r="F15" s="39" t="s">
-        <v>255</v>
+      <c r="F15" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="32" t="s">
         <v>106</v>
       </c>
-      <c r="B16" s="40" t="s">
+      <c r="B16" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="33" t="s">
-        <v>262</v>
-      </c>
-      <c r="D16" s="33" t="s">
-        <v>269</v>
-      </c>
-      <c r="E16" s="34" t="s">
-        <v>263</v>
-      </c>
-      <c r="F16" s="35" t="s">
-        <v>255</v>
+      <c r="C16" s="34" t="s">
+        <v>267</v>
+      </c>
+      <c r="D16" s="34" t="s">
+        <v>274</v>
+      </c>
+      <c r="E16" s="35" t="s">
+        <v>268</v>
+      </c>
+      <c r="F16" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="B17" s="40" t="s">
+      <c r="B17" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="37" t="s">
-        <v>262</v>
-      </c>
-      <c r="D17" s="37" t="s">
-        <v>270</v>
-      </c>
-      <c r="E17" s="38" t="s">
-        <v>263</v>
-      </c>
-      <c r="F17" s="39" t="s">
-        <v>255</v>
+      <c r="C17" s="38" t="s">
+        <v>267</v>
+      </c>
+      <c r="D17" s="38" t="s">
+        <v>275</v>
+      </c>
+      <c r="E17" s="39" t="s">
+        <v>268</v>
+      </c>
+      <c r="F17" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="32" t="s">
         <v>116</v>
       </c>
-      <c r="B18" s="41" t="s">
+      <c r="B18" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="C18" s="33" t="s">
-        <v>271</v>
-      </c>
-      <c r="D18" s="33" t="s">
-        <v>272</v>
-      </c>
-      <c r="E18" s="34" t="s">
-        <v>273</v>
-      </c>
-      <c r="F18" s="35" t="s">
-        <v>255</v>
+      <c r="C18" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="D18" s="34" t="s">
+        <v>277</v>
+      </c>
+      <c r="E18" s="35" t="s">
+        <v>278</v>
+      </c>
+      <c r="F18" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="B19" s="41" t="s">
+      <c r="B19" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="C19" s="37" t="s">
-        <v>271</v>
-      </c>
-      <c r="D19" s="37" t="s">
-        <v>274</v>
-      </c>
-      <c r="E19" s="38" t="s">
-        <v>273</v>
-      </c>
-      <c r="F19" s="39" t="s">
-        <v>255</v>
+      <c r="C19" s="38" t="s">
+        <v>276</v>
+      </c>
+      <c r="D19" s="38" t="s">
+        <v>279</v>
+      </c>
+      <c r="E19" s="39" t="s">
+        <v>278</v>
+      </c>
+      <c r="F19" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="31" t="s">
+      <c r="A20" s="32" t="s">
         <v>127</v>
       </c>
-      <c r="B20" s="41" t="s">
+      <c r="B20" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="C20" s="33" t="s">
-        <v>271</v>
-      </c>
-      <c r="D20" s="33" t="s">
-        <v>275</v>
-      </c>
-      <c r="E20" s="34" t="s">
-        <v>273</v>
-      </c>
-      <c r="F20" s="35" t="s">
-        <v>255</v>
+      <c r="C20" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="D20" s="34" t="s">
+        <v>280</v>
+      </c>
+      <c r="E20" s="35" t="s">
+        <v>278</v>
+      </c>
+      <c r="F20" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="37" t="s">
         <v>132</v>
       </c>
-      <c r="B21" s="41" t="s">
+      <c r="B21" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="C21" s="37" t="s">
-        <v>271</v>
-      </c>
-      <c r="D21" s="37" t="s">
+      <c r="C21" s="38" t="s">
+        <v>276</v>
+      </c>
+      <c r="D21" s="38" t="s">
         <v>134</v>
       </c>
-      <c r="E21" s="38" t="s">
+      <c r="E21" s="39" t="s">
+        <v>281</v>
+      </c>
+      <c r="F21" s="40" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="32" t="s">
+        <v>138</v>
+      </c>
+      <c r="B22" s="42" t="s">
+        <v>117</v>
+      </c>
+      <c r="C22" s="34" t="s">
         <v>276</v>
       </c>
-      <c r="F21" s="39" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="31" t="s">
-        <v>138</v>
-      </c>
-      <c r="B22" s="41" t="s">
+      <c r="D22" s="34" t="s">
+        <v>282</v>
+      </c>
+      <c r="E22" s="35" t="s">
+        <v>283</v>
+      </c>
+      <c r="F22" s="36" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="37" t="s">
+        <v>145</v>
+      </c>
+      <c r="B23" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="C22" s="33" t="s">
-        <v>271</v>
-      </c>
-      <c r="D22" s="33" t="s">
-        <v>277</v>
-      </c>
-      <c r="E22" s="34" t="s">
+      <c r="C23" s="38" t="s">
+        <v>276</v>
+      </c>
+      <c r="D23" s="38" t="s">
+        <v>148</v>
+      </c>
+      <c r="E23" s="39" t="s">
         <v>278</v>
       </c>
-      <c r="F22" s="35" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="36" t="s">
-        <v>144</v>
-      </c>
-      <c r="B23" s="41" t="s">
+      <c r="F23" s="40" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="32" t="s">
+        <v>152</v>
+      </c>
+      <c r="B24" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="C23" s="37" t="s">
-        <v>271</v>
-      </c>
-      <c r="D23" s="37" t="s">
-        <v>147</v>
-      </c>
-      <c r="E23" s="38" t="s">
-        <v>273</v>
-      </c>
-      <c r="F23" s="39" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="B24" s="41" t="s">
+      <c r="C24" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="D24" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="E24" s="35" t="s">
+        <v>278</v>
+      </c>
+      <c r="F24" s="36" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="37" t="s">
+        <v>157</v>
+      </c>
+      <c r="B25" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="C24" s="33" t="s">
-        <v>271</v>
-      </c>
-      <c r="D24" s="33" t="s">
-        <v>153</v>
-      </c>
-      <c r="E24" s="34" t="s">
-        <v>273</v>
-      </c>
-      <c r="F24" s="35" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="36" t="s">
-        <v>156</v>
-      </c>
-      <c r="B25" s="41" t="s">
+      <c r="C25" s="38" t="s">
+        <v>276</v>
+      </c>
+      <c r="D25" s="38" t="s">
+        <v>159</v>
+      </c>
+      <c r="E25" s="39" t="s">
+        <v>281</v>
+      </c>
+      <c r="F25" s="40" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="32" t="s">
+        <v>163</v>
+      </c>
+      <c r="B26" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="C25" s="37" t="s">
-        <v>271</v>
-      </c>
-      <c r="D25" s="37" t="s">
-        <v>158</v>
-      </c>
-      <c r="E25" s="38" t="s">
+      <c r="C26" s="34" t="s">
         <v>276</v>
       </c>
-      <c r="F25" s="39" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="31" t="s">
-        <v>162</v>
-      </c>
-      <c r="B26" s="41" t="s">
-        <v>117</v>
-      </c>
-      <c r="C26" s="33" t="s">
-        <v>271</v>
-      </c>
-      <c r="D26" s="33" t="s">
-        <v>164</v>
-      </c>
-      <c r="E26" s="34" t="s">
-        <v>276</v>
-      </c>
-      <c r="F26" s="35" t="s">
-        <v>255</v>
+      <c r="D26" s="34" t="s">
+        <v>165</v>
+      </c>
+      <c r="E26" s="35" t="s">
+        <v>281</v>
+      </c>
+      <c r="F26" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="36" t="s">
-        <v>169</v>
-      </c>
-      <c r="B27" s="42" t="s">
+      <c r="A27" s="37" t="s">
         <v>170</v>
       </c>
-      <c r="C27" s="37" t="s">
-        <v>279</v>
-      </c>
-      <c r="D27" s="37" t="s">
-        <v>280</v>
-      </c>
-      <c r="E27" s="38" t="s">
-        <v>281</v>
-      </c>
-      <c r="F27" s="39" t="s">
-        <v>255</v>
+      <c r="B27" s="43" t="s">
+        <v>171</v>
+      </c>
+      <c r="C27" s="38" t="s">
+        <v>284</v>
+      </c>
+      <c r="D27" s="38" t="s">
+        <v>285</v>
+      </c>
+      <c r="E27" s="39" t="s">
+        <v>286</v>
+      </c>
+      <c r="F27" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="31" t="s">
-        <v>178</v>
-      </c>
-      <c r="B28" s="42" t="s">
-        <v>170</v>
-      </c>
-      <c r="C28" s="33" t="s">
-        <v>279</v>
-      </c>
-      <c r="D28" s="33" t="s">
-        <v>282</v>
-      </c>
-      <c r="E28" s="34" t="s">
-        <v>281</v>
-      </c>
-      <c r="F28" s="35" t="s">
-        <v>255</v>
+      <c r="A28" s="32" t="s">
+        <v>179</v>
+      </c>
+      <c r="B28" s="43" t="s">
+        <v>171</v>
+      </c>
+      <c r="C28" s="34" t="s">
+        <v>284</v>
+      </c>
+      <c r="D28" s="34" t="s">
+        <v>287</v>
+      </c>
+      <c r="E28" s="35" t="s">
+        <v>286</v>
+      </c>
+      <c r="F28" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="36" t="s">
-        <v>183</v>
-      </c>
-      <c r="B29" s="42" t="s">
-        <v>170</v>
-      </c>
-      <c r="C29" s="37" t="s">
-        <v>279</v>
-      </c>
-      <c r="D29" s="37" t="s">
-        <v>283</v>
-      </c>
-      <c r="E29" s="38" t="s">
-        <v>281</v>
-      </c>
-      <c r="F29" s="39" t="s">
-        <v>255</v>
+      <c r="A29" s="37" t="s">
+        <v>184</v>
+      </c>
+      <c r="B29" s="43" t="s">
+        <v>171</v>
+      </c>
+      <c r="C29" s="38" t="s">
+        <v>284</v>
+      </c>
+      <c r="D29" s="38" t="s">
+        <v>288</v>
+      </c>
+      <c r="E29" s="39" t="s">
+        <v>286</v>
+      </c>
+      <c r="F29" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="31" t="s">
-        <v>188</v>
-      </c>
-      <c r="B30" s="42" t="s">
-        <v>170</v>
-      </c>
-      <c r="C30" s="33" t="s">
-        <v>279</v>
-      </c>
-      <c r="D30" s="33" t="s">
+      <c r="A30" s="32" t="s">
+        <v>189</v>
+      </c>
+      <c r="B30" s="43" t="s">
+        <v>171</v>
+      </c>
+      <c r="C30" s="34" t="s">
         <v>284</v>
       </c>
-      <c r="E30" s="34" t="s">
-        <v>281</v>
-      </c>
-      <c r="F30" s="35" t="s">
-        <v>255</v>
+      <c r="D30" s="34" t="s">
+        <v>289</v>
+      </c>
+      <c r="E30" s="35" t="s">
+        <v>286</v>
+      </c>
+      <c r="F30" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="36" t="s">
-        <v>194</v>
-      </c>
-      <c r="B31" s="42" t="s">
-        <v>170</v>
-      </c>
-      <c r="C31" s="37" t="s">
-        <v>279</v>
-      </c>
-      <c r="D31" s="37" t="s">
-        <v>196</v>
-      </c>
-      <c r="E31" s="38" t="s">
-        <v>285</v>
-      </c>
-      <c r="F31" s="39" t="s">
-        <v>255</v>
+      <c r="A31" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="B31" s="43" t="s">
+        <v>171</v>
+      </c>
+      <c r="C31" s="38" t="s">
+        <v>284</v>
+      </c>
+      <c r="D31" s="38" t="s">
+        <v>197</v>
+      </c>
+      <c r="E31" s="39" t="s">
+        <v>290</v>
+      </c>
+      <c r="F31" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="31" t="s">
-        <v>200</v>
-      </c>
-      <c r="B32" s="43" t="s">
+      <c r="A32" s="32" t="s">
         <v>201</v>
       </c>
-      <c r="C32" s="33" t="s">
-        <v>286</v>
-      </c>
-      <c r="D32" s="33" t="s">
-        <v>203</v>
-      </c>
-      <c r="E32" s="34" t="s">
-        <v>287</v>
-      </c>
-      <c r="F32" s="35" t="s">
-        <v>255</v>
+      <c r="B32" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="C32" s="34" t="s">
+        <v>291</v>
+      </c>
+      <c r="D32" s="34" t="s">
+        <v>204</v>
+      </c>
+      <c r="E32" s="35" t="s">
+        <v>292</v>
+      </c>
+      <c r="F32" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="36" t="s">
-        <v>207</v>
-      </c>
-      <c r="B33" s="43" t="s">
-        <v>201</v>
-      </c>
-      <c r="C33" s="37" t="s">
-        <v>286</v>
-      </c>
-      <c r="D33" s="37" t="s">
+      <c r="A33" s="37" t="s">
         <v>208</v>
       </c>
-      <c r="E33" s="38" t="s">
-        <v>287</v>
-      </c>
-      <c r="F33" s="39" t="s">
-        <v>255</v>
+      <c r="B33" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="C33" s="38" t="s">
+        <v>291</v>
+      </c>
+      <c r="D33" s="38" t="s">
+        <v>209</v>
+      </c>
+      <c r="E33" s="39" t="s">
+        <v>292</v>
+      </c>
+      <c r="F33" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="31" t="s">
-        <v>210</v>
-      </c>
-      <c r="B34" s="43" t="s">
-        <v>201</v>
-      </c>
-      <c r="C34" s="33" t="s">
-        <v>286</v>
-      </c>
-      <c r="D34" s="33" t="s">
-        <v>212</v>
-      </c>
-      <c r="E34" s="34" t="s">
-        <v>287</v>
-      </c>
-      <c r="F34" s="35" t="s">
-        <v>255</v>
+      <c r="A34" s="32" t="s">
+        <v>211</v>
+      </c>
+      <c r="B34" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="C34" s="34" t="s">
+        <v>291</v>
+      </c>
+      <c r="D34" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="E34" s="35" t="s">
+        <v>292</v>
+      </c>
+      <c r="F34" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="36" t="s">
-        <v>216</v>
-      </c>
-      <c r="B35" s="43" t="s">
-        <v>201</v>
-      </c>
-      <c r="C35" s="37" t="s">
-        <v>286</v>
-      </c>
-      <c r="D35" s="37" t="s">
+      <c r="A35" s="37" t="s">
         <v>217</v>
       </c>
-      <c r="E35" s="38" t="s">
-        <v>287</v>
-      </c>
-      <c r="F35" s="39" t="s">
-        <v>255</v>
+      <c r="B35" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="C35" s="38" t="s">
+        <v>291</v>
+      </c>
+      <c r="D35" s="38" t="s">
+        <v>218</v>
+      </c>
+      <c r="E35" s="39" t="s">
+        <v>292</v>
+      </c>
+      <c r="F35" s="40" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="31" t="s">
-        <v>221</v>
-      </c>
-      <c r="B36" s="43" t="s">
-        <v>201</v>
-      </c>
-      <c r="C36" s="33" t="s">
-        <v>286</v>
-      </c>
-      <c r="D36" s="33" t="s">
+      <c r="A36" s="32" t="s">
         <v>222</v>
       </c>
-      <c r="E36" s="34" t="s">
-        <v>287</v>
-      </c>
-      <c r="F36" s="35" t="s">
-        <v>255</v>
+      <c r="B36" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="C36" s="34" t="s">
+        <v>291</v>
+      </c>
+      <c r="D36" s="34" t="s">
+        <v>223</v>
+      </c>
+      <c r="E36" s="35" t="s">
+        <v>292</v>
+      </c>
+      <c r="F36" s="36" t="s">
+        <v>260</v>
       </c>
     </row>
   </sheetData>
@@ -4824,7 +4881,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -4834,206 +4891,235 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>288</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
+      <c r="A1" s="18" t="s">
+        <v>293</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
     </row>
     <row r="3" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
-        <v>289</v>
-      </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="A3" s="19" t="s">
+        <v>294</v>
+      </c>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="44" t="s">
-        <v>290</v>
-      </c>
-      <c r="B4" s="44" t="s">
-        <v>228</v>
-      </c>
-      <c r="C4" s="44" t="s">
-        <v>291</v>
-      </c>
-      <c r="D4" s="44" t="s">
-        <v>292</v>
-      </c>
-      <c r="E4" s="44" t="s">
-        <v>293</v>
-      </c>
-      <c r="F4" s="44" t="s">
-        <v>294</v>
+      <c r="A4" s="45" t="s">
+        <v>295</v>
+      </c>
+      <c r="B4" s="45" t="s">
+        <v>229</v>
+      </c>
+      <c r="C4" s="45" t="s">
+        <v>296</v>
+      </c>
+      <c r="D4" s="45" t="s">
+        <v>297</v>
+      </c>
+      <c r="E4" s="45" t="s">
+        <v>298</v>
+      </c>
+      <c r="F4" s="45" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="45" t="n">
+      <c r="A5" s="46" t="n">
         <f aca="false">COUNTIF('Test Cases'!A5:A41,"TC-*")</f>
         <v>33</v>
       </c>
-      <c r="B5" s="46" t="n">
+      <c r="B5" s="47" t="n">
         <f aca="false">COUNTIF('Test Cases'!A5:A41,"TC-*")</f>
         <v>33</v>
       </c>
-      <c r="C5" s="45" t="s">
-        <v>245</v>
-      </c>
-      <c r="D5" s="45" t="s">
-        <v>247</v>
-      </c>
-      <c r="E5" s="45" t="n">
+      <c r="C5" s="46" t="s">
+        <v>246</v>
+      </c>
+      <c r="D5" s="46" t="s">
+        <v>248</v>
+      </c>
+      <c r="E5" s="46" t="n">
         <f aca="false">COUNTIF('Test Cases'!B5:B41,"Y")</f>
         <v>4</v>
       </c>
-      <c r="F5" s="45" t="n">
+      <c r="F5" s="46" t="n">
         <f aca="false">COUNTIF('Test Cases'!D5:D41,"Y")</f>
         <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
-        <v>295</v>
-      </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
+      <c r="A7" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="B7" s="19"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="19" t="s">
-        <v>234</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>296</v>
-      </c>
-      <c r="D8" s="19" t="s">
+      <c r="B8" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>301</v>
+      </c>
+      <c r="D8" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="19" t="s">
-        <v>234</v>
-      </c>
-      <c r="F8" s="19" t="s">
-        <v>296</v>
+      <c r="E8" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="F8" s="20" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="21" t="n">
+      <c r="B9" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Functional")</f>
         <v>6</v>
       </c>
-      <c r="C9" s="21" t="str">
+      <c r="C9" s="22" t="str">
         <f aca="false">TEXT(B9/COUNTIF('Test Cases'!A5:A41,"TC-*"),"0%")</f>
         <v>18%</v>
       </c>
-      <c r="D9" s="25" t="s">
-        <v>170</v>
-      </c>
-      <c r="E9" s="21" t="n">
+      <c r="D9" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="E9" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Access Control")</f>
         <v>5</v>
       </c>
-      <c r="F9" s="21" t="str">
+      <c r="F9" s="22" t="str">
         <f aca="false">TEXT(E9/COUNTIF('Test Cases'!A5:A41,"TC-*"),"0%")</f>
         <v>15%</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="B10" s="21" t="n">
+      <c r="B10" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Boundary")</f>
         <v>8</v>
       </c>
-      <c r="C10" s="21" t="str">
+      <c r="C10" s="22" t="str">
         <f aca="false">TEXT(B10/COUNTIF('Test Cases'!A5:A41,"TC-*"),"0%")</f>
         <v>24%</v>
       </c>
-      <c r="D10" s="26" t="s">
-        <v>201</v>
-      </c>
-      <c r="E10" s="21" t="n">
+      <c r="D10" s="27" t="s">
+        <v>202</v>
+      </c>
+      <c r="E10" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Performance")</f>
         <v>5</v>
       </c>
-      <c r="F10" s="21" t="str">
+      <c r="F10" s="22" t="str">
         <f aca="false">TEXT(E10/COUNTIF('Test Cases'!A5:A41,"TC-*"),"0%")</f>
         <v>15%</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
+      <c r="A11" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="21" t="n">
+      <c r="B11" s="22" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Security")</f>
         <v>9</v>
       </c>
-      <c r="C11" s="21" t="str">
+      <c r="C11" s="22" t="str">
         <f aca="false">TEXT(B11/COUNTIF('Test Cases'!A5:A41,"TC-*"),"0%")</f>
         <v>27%</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
-        <v>297</v>
-      </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
+      <c r="A13" s="19" t="s">
+        <v>302</v>
+      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="19" t="s">
-        <v>234</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>298</v>
-      </c>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="B14" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>303</v>
+      </c>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="47" t="s">
+      <c r="A15" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="21" t="n">
-        <f aca="false">COUNTIF('Test Cases'!O5:O41,"Not Run")</f>
-        <v>33</v>
-      </c>
-      <c r="C15" s="48" t="s">
-        <v>299</v>
-      </c>
-      <c r="D15" s="48"/>
-      <c r="E15" s="48"/>
-      <c r="F15" s="48"/>
+      <c r="B15" s="22" t="n">
+        <f aca="false">COUNTIF('Test Cases'!O5:O41,"Pass")</f>
+        <v>32</v>
+      </c>
+      <c r="C15" s="49" t="s">
+        <v>304</v>
+      </c>
+      <c r="D15" s="49"/>
+      <c r="E15" s="49"/>
+      <c r="F15" s="49"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="50" t="s">
+        <v>143</v>
+      </c>
+      <c r="B16" s="22" t="n">
+        <f aca="false">COUNTIF('Test Cases'!O5:O41,"Observation")</f>
+        <v>1</v>
+      </c>
+      <c r="C16" s="49" t="s">
+        <v>305</v>
+      </c>
+      <c r="D16" s="49"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="49"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="28" t="s">
+        <v>306</v>
+      </c>
+      <c r="B17" s="51" t="s">
+        <v>307</v>
+      </c>
+      <c r="C17" s="51"/>
+      <c r="D17" s="51"/>
+      <c r="E17" s="51"/>
+      <c r="F17" s="51"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="C15:F15"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="B17:F17"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5058,245 +5144,245 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>300</v>
-      </c>
-      <c r="B1" s="17"/>
+      <c r="A1" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="B1" s="18"/>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="49" t="s">
-        <v>301</v>
-      </c>
-      <c r="B2" s="49"/>
+      <c r="A2" s="52" t="s">
+        <v>309</v>
+      </c>
+      <c r="B2" s="52"/>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="50" t="s">
-        <v>302</v>
-      </c>
-      <c r="B3" s="51" t="s">
-        <v>303</v>
+      <c r="A3" s="53" t="s">
+        <v>310</v>
+      </c>
+      <c r="B3" s="54" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="50" t="s">
-        <v>304</v>
-      </c>
-      <c r="B4" s="51" t="s">
-        <v>305</v>
+      <c r="A4" s="53" t="s">
+        <v>312</v>
+      </c>
+      <c r="B4" s="54" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="50" t="s">
-        <v>306</v>
-      </c>
-      <c r="B5" s="51" t="s">
-        <v>307</v>
+      <c r="A5" s="53" t="s">
+        <v>314</v>
+      </c>
+      <c r="B5" s="54" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="50" t="s">
-        <v>308</v>
-      </c>
-      <c r="B6" s="51" t="s">
-        <v>309</v>
+      <c r="A6" s="53" t="s">
+        <v>316</v>
+      </c>
+      <c r="B6" s="54" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="50" t="s">
-        <v>310</v>
-      </c>
-      <c r="B7" s="51" t="s">
-        <v>311</v>
+      <c r="A7" s="53" t="s">
+        <v>318</v>
+      </c>
+      <c r="B7" s="54" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="49" t="s">
-        <v>312</v>
-      </c>
-      <c r="B8" s="49"/>
+      <c r="A8" s="52" t="s">
+        <v>320</v>
+      </c>
+      <c r="B8" s="52"/>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="50" t="s">
-        <v>313</v>
-      </c>
-      <c r="B9" s="51" t="s">
-        <v>314</v>
+      <c r="A9" s="53" t="s">
+        <v>321</v>
+      </c>
+      <c r="B9" s="54" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="50" t="s">
+      <c r="A10" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="51" t="s">
-        <v>315</v>
+      <c r="B10" s="54" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="50" t="s">
+      <c r="A11" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="51" t="s">
-        <v>316</v>
+      <c r="B11" s="54" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="51" t="s">
-        <v>317</v>
+      <c r="B12" s="54" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="50" t="s">
+      <c r="A13" s="53" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="51" t="s">
-        <v>318</v>
+      <c r="B13" s="54" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="50" t="s">
+      <c r="A14" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="51" t="s">
-        <v>319</v>
+      <c r="B14" s="54" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="49" t="s">
-        <v>320</v>
-      </c>
-      <c r="B15" s="49"/>
+      <c r="A15" s="52" t="s">
+        <v>328</v>
+      </c>
+      <c r="B15" s="52"/>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="52" t="s">
-        <v>321</v>
-      </c>
-      <c r="B16" s="51" t="s">
-        <v>322</v>
+      <c r="A16" s="55" t="s">
+        <v>329</v>
+      </c>
+      <c r="B16" s="54" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="53" t="s">
-        <v>323</v>
-      </c>
-      <c r="B17" s="51" t="s">
-        <v>324</v>
+      <c r="A17" s="56" t="s">
+        <v>330</v>
+      </c>
+      <c r="B17" s="54" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="54" t="s">
-        <v>325</v>
-      </c>
-      <c r="B18" s="51" t="s">
-        <v>31</v>
+      <c r="A18" s="57" t="s">
+        <v>332</v>
+      </c>
+      <c r="B18" s="54" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="55" t="s">
-        <v>326</v>
-      </c>
-      <c r="B19" s="51" t="s">
-        <v>327</v>
+      <c r="A19" s="58" t="s">
+        <v>334</v>
+      </c>
+      <c r="B19" s="54" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="56" t="s">
-        <v>328</v>
-      </c>
-      <c r="B20" s="51" t="s">
-        <v>329</v>
+      <c r="A20" s="59" t="s">
+        <v>335</v>
+      </c>
+      <c r="B20" s="54" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="49" t="s">
-        <v>330</v>
-      </c>
-      <c r="B21" s="49"/>
+      <c r="A21" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="B21" s="52"/>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="50" t="s">
+      <c r="A22" s="53" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="51" t="s">
-        <v>331</v>
+      <c r="B22" s="54" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="53" t="s">
         <v>70</v>
       </c>
-      <c r="B23" s="51" t="s">
-        <v>332</v>
+      <c r="B23" s="54" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="50" t="s">
+      <c r="A24" s="53" t="s">
         <v>117</v>
       </c>
-      <c r="B24" s="51" t="s">
-        <v>333</v>
+      <c r="B24" s="54" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="50" t="s">
-        <v>170</v>
-      </c>
-      <c r="B25" s="51" t="s">
-        <v>334</v>
+      <c r="A25" s="53" t="s">
+        <v>171</v>
+      </c>
+      <c r="B25" s="54" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="50" t="s">
-        <v>201</v>
-      </c>
-      <c r="B26" s="51" t="s">
-        <v>335</v>
+      <c r="A26" s="53" t="s">
+        <v>202</v>
+      </c>
+      <c r="B26" s="54" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="49" t="s">
-        <v>336</v>
-      </c>
-      <c r="B27" s="49"/>
+      <c r="A27" s="52" t="s">
+        <v>343</v>
+      </c>
+      <c r="B27" s="52"/>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="50" t="s">
-        <v>337</v>
-      </c>
-      <c r="B28" s="51" t="s">
-        <v>338</v>
+      <c r="A28" s="53" t="s">
+        <v>344</v>
+      </c>
+      <c r="B28" s="54" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="50" t="s">
-        <v>339</v>
-      </c>
-      <c r="B29" s="51" t="s">
-        <v>340</v>
+      <c r="A29" s="53" t="s">
+        <v>346</v>
+      </c>
+      <c r="B29" s="54" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="50" t="s">
-        <v>341</v>
-      </c>
-      <c r="B30" s="51" t="s">
-        <v>342</v>
+      <c r="A30" s="53" t="s">
+        <v>348</v>
+      </c>
+      <c r="B30" s="54" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="49" t="s">
-        <v>343</v>
-      </c>
-      <c r="B31" s="49"/>
+      <c r="A31" s="52" t="s">
+        <v>350</v>
+      </c>
+      <c r="B31" s="52"/>
     </row>
     <row r="32" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="50" t="s">
-        <v>344</v>
-      </c>
-      <c r="B32" s="51" t="s">
-        <v>345</v>
+      <c r="A32" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="B32" s="54" t="s">
+        <v>352</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: use tick marks and content-fitted rows in the test workbook
</commit_message>
<xml_diff>
--- a/test-cases/ParaBank_Test_Cases.xlsx
+++ b/test-cases/ParaBank_Test_Cases.xlsx
@@ -86,7 +86,7 @@
     <t xml:space="preserve">TC-001</t>
   </si>
   <si>
-    <t xml:space="preserve">Y</t>
+    <t xml:space="preserve">✓</t>
   </si>
   <si>
     <t xml:space="preserve">-</t>
@@ -1046,10 +1046,10 @@
     <t xml:space="preserve">Smoke / Reg. / E2E</t>
   </si>
   <si>
-    <t xml:space="preserve">Y = the test case belongs to that suite; - = it does not.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y = the test case is automated. Every case in this suite is automated.</t>
+    <t xml:space="preserve">✓ = the test case belongs to that suite;  -  = it does not.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✓ = the test case is automated. Every case in this suite is automated.</t>
   </si>
   <si>
     <t xml:space="preserve">Functional, Boundary, Security, Access Control or Performance.</t>
@@ -1146,7 +1146,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1209,8 +1209,16 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FF1E7B34"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFB0B7C3"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1219,6 +1227,13 @@
       <b val="true"/>
       <sz val="8"/>
       <color rgb="FF404040"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1501,7 +1516,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="64">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1527,58 +1542,74 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1586,31 +1617,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1618,15 +1649,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1634,19 +1665,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1654,31 +1685,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1686,23 +1717,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1710,35 +1733,43 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="17" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="17" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1769,7 +1800,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
       <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FFD9E2F3"/>
       <rgbColor rgb="FF7030A0"/>
       <rgbColor rgb="FFFFF2CC"/>
       <rgbColor rgb="FFDDEBF7"/>
@@ -1789,7 +1820,7 @@
       <rgbColor rgb="FFE2EFDA"/>
       <rgbColor rgb="FFC6EFCE"/>
       <rgbColor rgb="FFFFEB9C"/>
-      <rgbColor rgb="FFD9E2F3"/>
+      <rgbColor rgb="FFB0B7C3"/>
       <rgbColor rgb="FFEAD1DC"/>
       <rgbColor rgb="FFE1D5E7"/>
       <rgbColor rgb="FFFFC7CE"/>
@@ -2122,7 +2153,7 @@
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
     </row>
-    <row r="5" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>19</v>
       </c>
@@ -2132,283 +2163,283 @@
       <c r="C5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="J5" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="L5" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M5" s="8" t="s">
+      <c r="M5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="N5" s="6" t="s">
+      <c r="N5" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="O5" s="9" t="s">
+      <c r="O5" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P5" s="8"/>
-    </row>
-    <row r="6" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="P5" s="9"/>
+    </row>
+    <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="11" t="s">
+      <c r="C6" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="7" t="s">
+      <c r="E6" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="G6" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="H6" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="I6" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="12" t="s">
+      <c r="J6" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="K6" s="12" t="s">
+      <c r="K6" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="L6" s="12" t="s">
+      <c r="L6" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="M6" s="12" t="s">
+      <c r="M6" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="N6" s="11" t="s">
+      <c r="N6" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="O6" s="9" t="s">
+      <c r="O6" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P6" s="12"/>
-    </row>
-    <row r="7" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P6" s="15"/>
+    </row>
+    <row r="7" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="J7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="K7" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="L7" s="8" t="s">
+      <c r="L7" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="M7" s="8" t="s">
+      <c r="M7" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="N7" s="6" t="s">
+      <c r="N7" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="O7" s="9" t="s">
+      <c r="O7" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P7" s="8"/>
-    </row>
-    <row r="8" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+      <c r="P7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8" s="7" t="s">
+      <c r="B8" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="G8" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="H8" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="I8" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="J8" s="12" t="s">
+      <c r="J8" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="K8" s="12" t="s">
+      <c r="K8" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="L8" s="12" t="s">
+      <c r="L8" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="M8" s="12" t="s">
+      <c r="M8" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="N8" s="11" t="s">
+      <c r="N8" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="O8" s="9" t="s">
+      <c r="O8" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P8" s="12"/>
-    </row>
-    <row r="9" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P8" s="15"/>
+    </row>
+    <row r="9" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="I9" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="J9" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="K9" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="L9" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="M9" s="8" t="s">
+      <c r="M9" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="N9" s="6" t="s">
+      <c r="N9" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="O9" s="9" t="s">
+      <c r="O9" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P9" s="8"/>
-    </row>
-    <row r="10" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="P9" s="9"/>
+    </row>
+    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" s="7" t="s">
+      <c r="C10" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="G10" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="H10" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="J10" s="12" t="s">
+      <c r="J10" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="K10" s="12" t="s">
+      <c r="K10" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="L10" s="12" t="s">
+      <c r="L10" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="M10" s="12" t="s">
+      <c r="M10" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="N10" s="11" t="s">
+      <c r="N10" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="O10" s="9" t="s">
+      <c r="O10" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P10" s="12"/>
+      <c r="P10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
@@ -2430,389 +2461,389 @@
       <c r="O11" s="4"/>
       <c r="P11" s="4"/>
     </row>
-    <row r="12" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="H12" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="I12" s="8" t="s">
+      <c r="I12" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="J12" s="8" t="s">
+      <c r="J12" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="K12" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="L12" s="8" t="s">
+      <c r="L12" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="M12" s="8" t="s">
+      <c r="M12" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="N12" s="6" t="s">
+      <c r="N12" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="O12" s="9" t="s">
+      <c r="O12" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P12" s="8"/>
-    </row>
-    <row r="13" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+      <c r="P12" s="9"/>
+    </row>
+    <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="11" t="s">
+      <c r="C13" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E13" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F13" s="13" t="s">
+      <c r="E13" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="G13" s="12" t="s">
+      <c r="G13" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="H13" s="12" t="s">
+      <c r="H13" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="I13" s="12" t="s">
+      <c r="I13" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="J13" s="12" t="s">
+      <c r="J13" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="K13" s="12" t="s">
+      <c r="K13" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="L13" s="12" t="s">
+      <c r="L13" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="M13" s="12" t="s">
+      <c r="M13" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="N13" s="11" t="s">
+      <c r="N13" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="O13" s="9" t="s">
+      <c r="O13" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P13" s="12"/>
-    </row>
-    <row r="14" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P13" s="15"/>
+    </row>
+    <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H14" s="8" t="s">
+      <c r="H14" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="I14" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="J14" s="8" t="s">
+      <c r="J14" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="K14" s="8" t="s">
+      <c r="K14" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="L14" s="8" t="s">
+      <c r="L14" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="M14" s="8" t="s">
+      <c r="M14" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="N14" s="6" t="s">
+      <c r="N14" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="O14" s="9" t="s">
+      <c r="O14" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P14" s="8"/>
-    </row>
-    <row r="15" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
+      <c r="P14" s="9"/>
+    </row>
+    <row r="15" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15" s="11" t="s">
+      <c r="C15" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F15" s="13" t="s">
+      <c r="E15" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="G15" s="12" t="s">
+      <c r="G15" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="H15" s="12" t="s">
+      <c r="H15" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="I15" s="12" t="s">
+      <c r="I15" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="J15" s="12" t="s">
+      <c r="J15" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="K15" s="12" t="s">
+      <c r="K15" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="L15" s="12" t="s">
+      <c r="L15" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="M15" s="12" t="s">
+      <c r="M15" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="N15" s="11" t="s">
+      <c r="N15" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="O15" s="9" t="s">
+      <c r="O15" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P15" s="12"/>
-    </row>
-    <row r="16" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P15" s="15"/>
+    </row>
+    <row r="16" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F16" s="13" t="s">
+      <c r="F16" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G16" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="I16" s="8" t="s">
+      <c r="I16" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J16" s="8" t="s">
+      <c r="J16" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="K16" s="8" t="s">
+      <c r="K16" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="L16" s="8" t="s">
+      <c r="L16" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="M16" s="8" t="s">
+      <c r="M16" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="N16" s="6" t="s">
+      <c r="N16" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="O16" s="9" t="s">
+      <c r="O16" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P16" s="8"/>
-    </row>
-    <row r="17" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
+      <c r="P16" s="9"/>
+    </row>
+    <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D17" s="11" t="s">
+      <c r="C17" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E17" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F17" s="13" t="s">
+      <c r="E17" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F17" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="G17" s="12" t="s">
+      <c r="G17" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="H17" s="12" t="s">
+      <c r="H17" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="I17" s="12" t="s">
+      <c r="I17" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="J17" s="12" t="s">
+      <c r="J17" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="K17" s="12" t="s">
+      <c r="K17" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="L17" s="12" t="s">
+      <c r="L17" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="M17" s="12" t="s">
+      <c r="M17" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="N17" s="11" t="s">
+      <c r="N17" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="O17" s="9" t="s">
+      <c r="O17" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P17" s="12"/>
-    </row>
-    <row r="18" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P17" s="15"/>
+    </row>
+    <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F18" s="13" t="s">
+      <c r="F18" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="G18" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="H18" s="8" t="s">
+      <c r="H18" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="I18" s="8" t="s">
+      <c r="I18" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="J18" s="8" t="s">
+      <c r="J18" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="K18" s="8" t="s">
+      <c r="K18" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="L18" s="8" t="s">
+      <c r="L18" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="M18" s="8" t="s">
+      <c r="M18" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="N18" s="6" t="s">
+      <c r="N18" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="O18" s="9" t="s">
+      <c r="O18" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P18" s="8"/>
-    </row>
-    <row r="19" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
+      <c r="P18" s="9"/>
+    </row>
+    <row r="19" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D19" s="11" t="s">
+      <c r="C19" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E19" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F19" s="13" t="s">
+      <c r="E19" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="G19" s="12" t="s">
+      <c r="G19" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="H19" s="12" t="s">
+      <c r="H19" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="I19" s="12" t="s">
+      <c r="I19" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="J19" s="12" t="s">
+      <c r="J19" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="K19" s="12" t="s">
+      <c r="K19" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="L19" s="12" t="s">
+      <c r="L19" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="M19" s="12" t="s">
+      <c r="M19" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="N19" s="11" t="s">
+      <c r="N19" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="O19" s="9" t="s">
+      <c r="O19" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P19" s="12"/>
+      <c r="P19" s="15"/>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
@@ -2834,301 +2865,301 @@
       <c r="O20" s="4"/>
       <c r="P20" s="4"/>
     </row>
-    <row r="21" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="F21" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H21" s="8" t="s">
+      <c r="H21" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="I21" s="8" t="s">
+      <c r="I21" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="J21" s="8" t="s">
+      <c r="J21" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="K21" s="8" t="s">
+      <c r="K21" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="L21" s="8" t="s">
+      <c r="L21" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="M21" s="8" t="s">
+      <c r="M21" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="N21" s="6" t="s">
+      <c r="N21" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="O21" s="9" t="s">
+      <c r="O21" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P21" s="8"/>
-    </row>
-    <row r="22" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="s">
+      <c r="P21" s="9"/>
+    </row>
+    <row r="22" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D22" s="11" t="s">
+      <c r="C22" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E22" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F22" s="14" t="s">
+      <c r="E22" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F22" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="G22" s="12" t="s">
+      <c r="G22" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="H22" s="12" t="s">
+      <c r="H22" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="I22" s="12" t="s">
+      <c r="I22" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="J22" s="12" t="s">
+      <c r="J22" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="K22" s="12" t="s">
+      <c r="K22" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="L22" s="12" t="s">
+      <c r="L22" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="M22" s="12" t="s">
+      <c r="M22" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="N22" s="11" t="s">
+      <c r="N22" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="O22" s="9" t="s">
+      <c r="O22" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P22" s="12"/>
-    </row>
-    <row r="23" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P22" s="15"/>
+    </row>
+    <row r="23" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F23" s="14" t="s">
+      <c r="F23" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="G23" s="8" t="s">
+      <c r="G23" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="8" t="s">
+      <c r="H23" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="I23" s="8" t="s">
+      <c r="I23" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="J23" s="8" t="s">
+      <c r="J23" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="K23" s="8" t="s">
+      <c r="K23" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="L23" s="8" t="s">
+      <c r="L23" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="M23" s="8" t="s">
+      <c r="M23" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="N23" s="6" t="s">
+      <c r="N23" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="O23" s="9" t="s">
+      <c r="O23" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P23" s="8"/>
-    </row>
-    <row r="24" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
+      <c r="P23" s="9"/>
+    </row>
+    <row r="24" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="B24" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D24" s="11" t="s">
+      <c r="B24" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F24" s="14" t="s">
+      <c r="E24" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F24" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="G24" s="12" t="s">
+      <c r="G24" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="H24" s="12" t="s">
+      <c r="H24" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="I24" s="12" t="s">
+      <c r="I24" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="J24" s="12" t="s">
+      <c r="J24" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="K24" s="12" t="s">
+      <c r="K24" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="L24" s="12" t="s">
+      <c r="L24" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="M24" s="12" t="s">
+      <c r="M24" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="N24" s="11" t="s">
+      <c r="N24" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="O24" s="9" t="s">
+      <c r="O24" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P24" s="12"/>
-    </row>
-    <row r="25" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P24" s="15"/>
+    </row>
+    <row r="25" customFormat="false" ht="75.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="F25" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="G25" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H25" s="8" t="s">
+      <c r="H25" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="I25" s="8" t="s">
+      <c r="I25" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="J25" s="8" t="s">
+      <c r="J25" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="K25" s="8" t="s">
+      <c r="K25" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="L25" s="8" t="s">
+      <c r="L25" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="M25" s="8" t="s">
+      <c r="M25" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="N25" s="6" t="s">
+      <c r="N25" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="O25" s="15" t="s">
+      <c r="O25" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="P25" s="8" t="s">
+      <c r="P25" s="9" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="s">
+    <row r="26" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="B26" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C26" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D26" s="11" t="s">
+      <c r="B26" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E26" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F26" s="14" t="s">
+      <c r="E26" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F26" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="G26" s="12" t="s">
+      <c r="G26" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="H26" s="12" t="s">
+      <c r="H26" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="I26" s="12" t="s">
+      <c r="I26" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="J26" s="12" t="s">
+      <c r="J26" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="K26" s="12" t="s">
+      <c r="K26" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="L26" s="12" t="s">
+      <c r="L26" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="M26" s="12" t="s">
+      <c r="M26" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="N26" s="11" t="s">
+      <c r="N26" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="O26" s="9" t="s">
+      <c r="O26" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P26" s="12"/>
-    </row>
-    <row r="27" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P26" s="15"/>
+    </row>
+    <row r="27" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C27" s="6" t="s">
@@ -3140,133 +3171,133 @@
       <c r="E27" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F27" s="14" t="s">
+      <c r="F27" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="G27" s="8" t="s">
+      <c r="G27" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="H27" s="8" t="s">
+      <c r="H27" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="I27" s="8" t="s">
+      <c r="I27" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="J27" s="8" t="s">
+      <c r="J27" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="K27" s="8" t="s">
+      <c r="K27" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="L27" s="8" t="s">
+      <c r="L27" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="M27" s="8" t="s">
+      <c r="M27" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="N27" s="6" t="s">
+      <c r="N27" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="O27" s="9" t="s">
+      <c r="O27" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P27" s="8"/>
-    </row>
-    <row r="28" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="s">
+      <c r="P27" s="9"/>
+    </row>
+    <row r="28" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C28" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E28" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F28" s="14" t="s">
+      <c r="C28" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F28" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="G28" s="12" t="s">
+      <c r="G28" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="H28" s="12" t="s">
+      <c r="H28" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="I28" s="12" t="s">
+      <c r="I28" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="J28" s="12" t="s">
+      <c r="J28" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="K28" s="12" t="s">
+      <c r="K28" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="L28" s="12" t="s">
+      <c r="L28" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="M28" s="12" t="s">
+      <c r="M28" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="N28" s="11" t="s">
+      <c r="N28" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="O28" s="9" t="s">
+      <c r="O28" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P28" s="12"/>
-    </row>
-    <row r="29" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P28" s="15"/>
+    </row>
+    <row r="29" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F29" s="14" t="s">
+      <c r="F29" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="G29" s="8" t="s">
+      <c r="G29" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="H29" s="8" t="s">
+      <c r="H29" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="I29" s="8" t="s">
+      <c r="I29" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="J29" s="8" t="s">
+      <c r="J29" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="K29" s="8" t="s">
+      <c r="K29" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="L29" s="8" t="s">
+      <c r="L29" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="M29" s="8" t="s">
+      <c r="M29" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="N29" s="6" t="s">
+      <c r="N29" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="O29" s="9" t="s">
+      <c r="O29" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P29" s="8"/>
+      <c r="P29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
@@ -3288,155 +3319,155 @@
       <c r="O30" s="4"/>
       <c r="P30" s="4"/>
     </row>
-    <row r="31" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10" t="s">
+    <row r="31" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12" t="s">
         <v>170</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C31" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D31" s="11" t="s">
+      <c r="C31" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F31" s="16" t="s">
+      <c r="E31" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F31" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="G31" s="12" t="s">
+      <c r="G31" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="H31" s="12" t="s">
+      <c r="H31" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="I31" s="12" t="s">
+      <c r="I31" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="J31" s="12" t="s">
+      <c r="J31" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="K31" s="12" t="s">
+      <c r="K31" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="L31" s="12" t="s">
+      <c r="L31" s="15" t="s">
         <v>177</v>
       </c>
-      <c r="M31" s="12" t="s">
+      <c r="M31" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="N31" s="11" t="s">
+      <c r="N31" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="O31" s="9" t="s">
+      <c r="O31" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P31" s="12"/>
-    </row>
-    <row r="32" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P31" s="15"/>
+    </row>
+    <row r="32" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F32" s="16" t="s">
+      <c r="F32" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="G32" s="8" t="s">
+      <c r="G32" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="H32" s="8" t="s">
+      <c r="H32" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="I32" s="8" t="s">
+      <c r="I32" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="J32" s="8" t="s">
+      <c r="J32" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="K32" s="8" t="s">
+      <c r="K32" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="L32" s="8" t="s">
+      <c r="L32" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="M32" s="8" t="s">
+      <c r="M32" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="N32" s="6" t="s">
+      <c r="N32" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="O32" s="9" t="s">
+      <c r="O32" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P32" s="8"/>
-    </row>
-    <row r="33" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10" t="s">
+      <c r="P32" s="9"/>
+    </row>
+    <row r="33" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C33" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D33" s="11" t="s">
+      <c r="C33" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E33" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F33" s="16" t="s">
+      <c r="E33" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F33" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="G33" s="12" t="s">
+      <c r="G33" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="H33" s="12" t="s">
+      <c r="H33" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="I33" s="12" t="s">
+      <c r="I33" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="J33" s="12" t="s">
+      <c r="J33" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="K33" s="12" t="s">
+      <c r="K33" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="L33" s="12" t="s">
+      <c r="L33" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="M33" s="12" t="s">
+      <c r="M33" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="N33" s="11" t="s">
+      <c r="N33" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="O33" s="9" t="s">
+      <c r="O33" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P33" s="12"/>
-    </row>
-    <row r="34" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P33" s="15"/>
+    </row>
+    <row r="34" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C34" s="6" t="s">
@@ -3448,85 +3479,85 @@
       <c r="E34" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F34" s="16" t="s">
+      <c r="F34" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="G34" s="8" t="s">
+      <c r="G34" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="H34" s="8" t="s">
+      <c r="H34" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="I34" s="8" t="s">
+      <c r="I34" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="J34" s="8" t="s">
+      <c r="J34" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="K34" s="8" t="s">
+      <c r="K34" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="L34" s="8" t="s">
+      <c r="L34" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="M34" s="8" t="s">
+      <c r="M34" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="N34" s="6" t="s">
+      <c r="N34" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="O34" s="9" t="s">
+      <c r="O34" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P34" s="8"/>
-    </row>
-    <row r="35" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10" t="s">
+      <c r="P34" s="9"/>
+    </row>
+    <row r="35" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C35" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D35" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E35" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F35" s="16" t="s">
+      <c r="C35" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F35" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="G35" s="12" t="s">
+      <c r="G35" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="H35" s="12" t="s">
+      <c r="H35" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="I35" s="12" t="s">
+      <c r="I35" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="J35" s="12" t="s">
+      <c r="J35" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="K35" s="12" t="s">
+      <c r="K35" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="L35" s="12" t="s">
+      <c r="L35" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="M35" s="12" t="s">
+      <c r="M35" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="N35" s="11" t="s">
+      <c r="N35" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="O35" s="9" t="s">
+      <c r="O35" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P35" s="12"/>
+      <c r="P35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
@@ -3548,107 +3579,107 @@
       <c r="O36" s="4"/>
       <c r="P36" s="4"/>
     </row>
-    <row r="37" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D37" s="6" t="s">
+      <c r="D37" s="7" t="s">
         <v>21</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F37" s="17" t="s">
+      <c r="F37" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="G37" s="8" t="s">
+      <c r="G37" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="H37" s="8" t="s">
+      <c r="H37" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="I37" s="8" t="s">
+      <c r="I37" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="J37" s="8" t="s">
+      <c r="J37" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="K37" s="8" t="s">
+      <c r="K37" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="L37" s="8" t="s">
+      <c r="L37" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="M37" s="8" t="s">
+      <c r="M37" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="N37" s="6" t="s">
+      <c r="N37" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="O37" s="9" t="s">
+      <c r="O37" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P37" s="8"/>
-    </row>
-    <row r="38" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="10" t="s">
+      <c r="P37" s="9"/>
+    </row>
+    <row r="38" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="12" t="s">
         <v>208</v>
       </c>
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C38" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D38" s="11" t="s">
+      <c r="C38" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D38" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E38" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F38" s="17" t="s">
+      <c r="E38" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F38" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="G38" s="12" t="s">
+      <c r="G38" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="H38" s="12" t="s">
+      <c r="H38" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="I38" s="12" t="s">
+      <c r="I38" s="15" t="s">
         <v>209</v>
       </c>
-      <c r="J38" s="12" t="s">
+      <c r="J38" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="K38" s="12" t="s">
+      <c r="K38" s="15" t="s">
         <v>210</v>
       </c>
-      <c r="L38" s="12" t="s">
+      <c r="L38" s="15" t="s">
         <v>206</v>
       </c>
-      <c r="M38" s="12" t="s">
+      <c r="M38" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="N38" s="11" t="s">
+      <c r="N38" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="O38" s="9" t="s">
+      <c r="O38" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P38" s="12"/>
-    </row>
-    <row r="39" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P38" s="15"/>
+    </row>
+    <row r="39" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C39" s="6" t="s">
@@ -3660,91 +3691,91 @@
       <c r="E39" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F39" s="17" t="s">
+      <c r="F39" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="G39" s="8" t="s">
+      <c r="G39" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H39" s="8" t="s">
+      <c r="H39" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="I39" s="8" t="s">
+      <c r="I39" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="J39" s="8" t="s">
+      <c r="J39" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="K39" s="8" t="s">
+      <c r="K39" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="L39" s="8" t="s">
+      <c r="L39" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="M39" s="8" t="s">
+      <c r="M39" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="N39" s="6" t="s">
+      <c r="N39" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="O39" s="9" t="s">
+      <c r="O39" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P39" s="8"/>
-    </row>
-    <row r="40" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="10" t="s">
+      <c r="P39" s="9"/>
+    </row>
+    <row r="40" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="12" t="s">
         <v>217</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C40" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D40" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E40" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F40" s="17" t="s">
+      <c r="C40" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E40" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F40" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="G40" s="12" t="s">
+      <c r="G40" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="H40" s="12" t="s">
+      <c r="H40" s="15" t="s">
         <v>212</v>
       </c>
-      <c r="I40" s="12" t="s">
+      <c r="I40" s="15" t="s">
         <v>218</v>
       </c>
-      <c r="J40" s="12" t="s">
+      <c r="J40" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="K40" s="12" t="s">
+      <c r="K40" s="15" t="s">
         <v>219</v>
       </c>
-      <c r="L40" s="12" t="s">
+      <c r="L40" s="15" t="s">
         <v>220</v>
       </c>
-      <c r="M40" s="12" t="s">
+      <c r="M40" s="15" t="s">
         <v>221</v>
       </c>
-      <c r="N40" s="11" t="s">
+      <c r="N40" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="O40" s="9" t="s">
+      <c r="O40" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P40" s="12"/>
-    </row>
-    <row r="41" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P40" s="15"/>
+    </row>
+    <row r="41" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C41" s="6" t="s">
@@ -3756,37 +3787,37 @@
       <c r="E41" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F41" s="17" t="s">
+      <c r="F41" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="G41" s="8" t="s">
+      <c r="G41" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="H41" s="8" t="s">
+      <c r="H41" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="I41" s="8" t="s">
+      <c r="I41" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="J41" s="8" t="s">
+      <c r="J41" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="K41" s="8" t="s">
+      <c r="K41" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="L41" s="8" t="s">
+      <c r="L41" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="M41" s="8" t="s">
+      <c r="M41" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="N41" s="6" t="s">
+      <c r="N41" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="O41" s="9" t="s">
+      <c r="O41" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="P41" s="8"/>
+      <c r="P41" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -3821,310 +3852,310 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="22" t="s">
         <v>226</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
     </row>
     <row r="3" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="23" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="24" t="s">
         <v>228</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="24" t="s">
         <v>229</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="24" t="s">
         <v>230</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="24" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Functional")</f>
         <v>6</v>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Functional")</f>
         <v>6</v>
       </c>
-      <c r="D5" s="22" t="n">
+      <c r="D5" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="27" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Boundary")</f>
         <v>8</v>
       </c>
-      <c r="C6" s="22" t="n">
+      <c r="C6" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Boundary")</f>
         <v>8</v>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="D6" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="23" t="s">
+      <c r="E6" s="27" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="29" t="s">
         <v>117</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Security")</f>
         <v>9</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Security")</f>
         <v>9</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="27" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="26" t="s">
+      <c r="A8" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Access Control")</f>
         <v>5</v>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Access Control")</f>
         <v>5</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="23" t="s">
+      <c r="E8" s="27" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="31" t="s">
         <v>202</v>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Performance")</f>
         <v>5</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Performance")</f>
         <v>5</v>
       </c>
-      <c r="D9" s="22" t="n">
+      <c r="D9" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="27" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="B10" s="29" t="n">
+      <c r="B10" s="33" t="n">
         <f aca="false">SUM(B5:B9)</f>
         <v>33</v>
       </c>
-      <c r="C10" s="29" t="n">
+      <c r="C10" s="33" t="n">
         <f aca="false">SUM(C5:C9)</f>
         <v>33</v>
       </c>
-      <c r="D10" s="29" t="n">
+      <c r="D10" s="33" t="n">
         <f aca="false">SUM(D5:D9)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="30" t="s">
+      <c r="E10" s="34" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="23" t="s">
         <v>234</v>
       </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="24" t="s">
         <v>235</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="24" t="s">
         <v>236</v>
       </c>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="22" t="n">
+      <c r="B14" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!N5:N41,"P1 - High")</f>
         <v>7</v>
       </c>
-      <c r="C14" s="22" t="str">
+      <c r="C14" s="26" t="str">
         <f aca="false">TEXT(B14/B10,"0%")</f>
         <v>21%</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="22" t="n">
+      <c r="B15" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!N5:N41,"P2 - Medium")</f>
         <v>18</v>
       </c>
-      <c r="C15" s="22" t="str">
+      <c r="C15" s="26" t="str">
         <f aca="false">TEXT(B15/B10,"0%")</f>
         <v>55%</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="35" t="s">
         <v>89</v>
       </c>
-      <c r="B16" s="22" t="n">
+      <c r="B16" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!N5:N41,"P3 - Low")</f>
         <v>8</v>
       </c>
-      <c r="C16" s="22" t="str">
+      <c r="C16" s="26" t="str">
         <f aca="false">TEXT(B16/B10,"0%")</f>
         <v>24%</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="23" t="s">
         <v>237</v>
       </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="s">
+      <c r="A19" s="24" t="s">
         <v>238</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="24" t="s">
         <v>239</v>
       </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="31" t="s">
+      <c r="A20" s="35" t="s">
         <v>240</v>
       </c>
-      <c r="B20" s="22" t="n">
+      <c r="B20" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!A5:A41,"TC-*")</f>
         <v>33</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="31" t="s">
+      <c r="A21" s="35" t="s">
         <v>241</v>
       </c>
-      <c r="B21" s="22" t="n">
+      <c r="B21" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!A5:A41,"TC-*")</f>
         <v>33</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="31" t="s">
+      <c r="A22" s="35" t="s">
         <v>242</v>
       </c>
-      <c r="B22" s="22" t="n">
-        <f aca="false">COUNTIF('Test Cases'!B5:B41,"Y")</f>
+      <c r="B22" s="26" t="n">
+        <f aca="false">COUNTIF('Test Cases'!B5:B41,"✓")</f>
         <v>4</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="31" t="s">
+      <c r="A23" s="35" t="s">
         <v>243</v>
       </c>
-      <c r="B23" s="22" t="n">
-        <f aca="false">COUNTIF('Test Cases'!D5:D41,"Y")</f>
+      <c r="B23" s="26" t="n">
+        <f aca="false">COUNTIF('Test Cases'!D5:D41,"✓")</f>
         <v>9</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="31" t="s">
+      <c r="A24" s="35" t="s">
         <v>244</v>
       </c>
-      <c r="B24" s="22" t="n">
+      <c r="B24" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!A5:A41,"TC-*")</f>
         <v>33</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="35" t="s">
         <v>245</v>
       </c>
-      <c r="B25" s="22" t="s">
+      <c r="B25" s="26" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="31" t="s">
+      <c r="A26" s="35" t="s">
         <v>247</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="26" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="31" t="s">
+      <c r="A27" s="35" t="s">
         <v>249</v>
       </c>
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="26" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="31" t="s">
+      <c r="A28" s="35" t="s">
         <v>251</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="26" t="s">
         <v>252</v>
       </c>
     </row>
@@ -4162,14 +4193,14 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="22" t="s">
         <v>253</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -4182,682 +4213,682 @@
       <c r="F2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="24" t="s">
         <v>255</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="24" t="s">
         <v>256</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="24" t="s">
         <v>257</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="24" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C4" s="38" t="s">
         <v>258</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="D4" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="35" t="s">
+      <c r="E4" s="39" t="s">
         <v>259</v>
       </c>
-      <c r="F4" s="36" t="s">
+      <c r="F4" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="38" t="s">
+      <c r="C5" s="42" t="s">
         <v>258</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="D5" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="39" t="s">
+      <c r="E5" s="43" t="s">
         <v>261</v>
       </c>
-      <c r="F5" s="40" t="s">
+      <c r="F5" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="38" t="s">
         <v>258</v>
       </c>
-      <c r="D6" s="34" t="s">
+      <c r="D6" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="35" t="s">
+      <c r="E6" s="39" t="s">
         <v>261</v>
       </c>
-      <c r="F6" s="36" t="s">
+      <c r="F6" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="38" t="s">
+      <c r="C7" s="42" t="s">
         <v>262</v>
       </c>
-      <c r="D7" s="38" t="s">
+      <c r="D7" s="42" t="s">
         <v>263</v>
       </c>
-      <c r="E7" s="39" t="s">
+      <c r="E7" s="43" t="s">
         <v>264</v>
       </c>
-      <c r="F7" s="40" t="s">
+      <c r="F7" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="38" t="s">
         <v>262</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="35" t="s">
+      <c r="E8" s="39" t="s">
         <v>265</v>
       </c>
-      <c r="F8" s="36" t="s">
+      <c r="F8" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="38" t="s">
+      <c r="C9" s="42" t="s">
         <v>262</v>
       </c>
-      <c r="D9" s="38" t="s">
+      <c r="D9" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="39" t="s">
+      <c r="E9" s="43" t="s">
         <v>266</v>
       </c>
-      <c r="F9" s="40" t="s">
+      <c r="F9" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="45" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="34" t="s">
+      <c r="C10" s="38" t="s">
         <v>267</v>
       </c>
-      <c r="D10" s="34" t="s">
+      <c r="D10" s="38" t="s">
         <v>72</v>
       </c>
-      <c r="E10" s="35" t="s">
+      <c r="E10" s="39" t="s">
         <v>268</v>
       </c>
-      <c r="F10" s="36" t="s">
+      <c r="F10" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="37" t="s">
+      <c r="A11" s="41" t="s">
         <v>77</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="45" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="38" t="s">
+      <c r="C11" s="42" t="s">
         <v>267</v>
       </c>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="42" t="s">
         <v>79</v>
       </c>
-      <c r="E11" s="39" t="s">
+      <c r="E11" s="43" t="s">
         <v>268</v>
       </c>
-      <c r="F11" s="40" t="s">
+      <c r="F11" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="36" t="s">
         <v>83</v>
       </c>
-      <c r="B12" s="41" t="s">
+      <c r="B12" s="45" t="s">
         <v>70</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="38" t="s">
         <v>267</v>
       </c>
-      <c r="D12" s="34" t="s">
+      <c r="D12" s="38" t="s">
         <v>269</v>
       </c>
-      <c r="E12" s="35" t="s">
+      <c r="E12" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="F12" s="36" t="s">
+      <c r="F12" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="37" t="s">
+      <c r="A13" s="41" t="s">
         <v>90</v>
       </c>
-      <c r="B13" s="41" t="s">
+      <c r="B13" s="45" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="38" t="s">
+      <c r="C13" s="42" t="s">
         <v>267</v>
       </c>
-      <c r="D13" s="38" t="s">
+      <c r="D13" s="42" t="s">
         <v>271</v>
       </c>
-      <c r="E13" s="39" t="s">
+      <c r="E13" s="43" t="s">
         <v>270</v>
       </c>
-      <c r="F13" s="40" t="s">
+      <c r="F13" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="32" t="s">
+      <c r="A14" s="36" t="s">
         <v>95</v>
       </c>
-      <c r="B14" s="41" t="s">
+      <c r="B14" s="45" t="s">
         <v>70</v>
       </c>
-      <c r="C14" s="34" t="s">
+      <c r="C14" s="38" t="s">
         <v>267</v>
       </c>
-      <c r="D14" s="34" t="s">
+      <c r="D14" s="38" t="s">
         <v>272</v>
       </c>
-      <c r="E14" s="35" t="s">
+      <c r="E14" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="F14" s="36" t="s">
+      <c r="F14" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="37" t="s">
+      <c r="A15" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="B15" s="41" t="s">
+      <c r="B15" s="45" t="s">
         <v>70</v>
       </c>
-      <c r="C15" s="38" t="s">
+      <c r="C15" s="42" t="s">
         <v>267</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="42" t="s">
         <v>273</v>
       </c>
-      <c r="E15" s="39" t="s">
+      <c r="E15" s="43" t="s">
         <v>268</v>
       </c>
-      <c r="F15" s="40" t="s">
+      <c r="F15" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="36" t="s">
         <v>106</v>
       </c>
-      <c r="B16" s="41" t="s">
+      <c r="B16" s="45" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="34" t="s">
+      <c r="C16" s="38" t="s">
         <v>267</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="D16" s="38" t="s">
         <v>274</v>
       </c>
-      <c r="E16" s="35" t="s">
+      <c r="E16" s="39" t="s">
         <v>268</v>
       </c>
-      <c r="F16" s="36" t="s">
+      <c r="F16" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="37" t="s">
+      <c r="A17" s="41" t="s">
         <v>110</v>
       </c>
-      <c r="B17" s="41" t="s">
+      <c r="B17" s="45" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="38" t="s">
+      <c r="C17" s="42" t="s">
         <v>267</v>
       </c>
-      <c r="D17" s="38" t="s">
+      <c r="D17" s="42" t="s">
         <v>275</v>
       </c>
-      <c r="E17" s="39" t="s">
+      <c r="E17" s="43" t="s">
         <v>268</v>
       </c>
-      <c r="F17" s="40" t="s">
+      <c r="F17" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="32" t="s">
+      <c r="A18" s="36" t="s">
         <v>116</v>
       </c>
-      <c r="B18" s="42" t="s">
+      <c r="B18" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="C18" s="34" t="s">
+      <c r="C18" s="38" t="s">
         <v>276</v>
       </c>
-      <c r="D18" s="34" t="s">
+      <c r="D18" s="38" t="s">
         <v>277</v>
       </c>
-      <c r="E18" s="35" t="s">
+      <c r="E18" s="39" t="s">
         <v>278</v>
       </c>
-      <c r="F18" s="36" t="s">
+      <c r="F18" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="37" t="s">
+      <c r="A19" s="41" t="s">
         <v>123</v>
       </c>
-      <c r="B19" s="42" t="s">
+      <c r="B19" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="C19" s="38" t="s">
+      <c r="C19" s="42" t="s">
         <v>276</v>
       </c>
-      <c r="D19" s="38" t="s">
+      <c r="D19" s="42" t="s">
         <v>279</v>
       </c>
-      <c r="E19" s="39" t="s">
+      <c r="E19" s="43" t="s">
         <v>278</v>
       </c>
-      <c r="F19" s="40" t="s">
+      <c r="F19" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="32" t="s">
+      <c r="A20" s="36" t="s">
         <v>127</v>
       </c>
-      <c r="B20" s="42" t="s">
+      <c r="B20" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="C20" s="34" t="s">
+      <c r="C20" s="38" t="s">
         <v>276</v>
       </c>
-      <c r="D20" s="34" t="s">
+      <c r="D20" s="38" t="s">
         <v>280</v>
       </c>
-      <c r="E20" s="35" t="s">
+      <c r="E20" s="39" t="s">
         <v>278</v>
       </c>
-      <c r="F20" s="36" t="s">
+      <c r="F20" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="41" t="s">
         <v>132</v>
       </c>
-      <c r="B21" s="42" t="s">
+      <c r="B21" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="C21" s="38" t="s">
+      <c r="C21" s="42" t="s">
         <v>276</v>
       </c>
-      <c r="D21" s="38" t="s">
+      <c r="D21" s="42" t="s">
         <v>134</v>
       </c>
-      <c r="E21" s="39" t="s">
+      <c r="E21" s="43" t="s">
         <v>281</v>
       </c>
-      <c r="F21" s="40" t="s">
+      <c r="F21" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="32" t="s">
+      <c r="A22" s="36" t="s">
         <v>138</v>
       </c>
-      <c r="B22" s="42" t="s">
+      <c r="B22" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="C22" s="34" t="s">
+      <c r="C22" s="38" t="s">
         <v>276</v>
       </c>
-      <c r="D22" s="34" t="s">
+      <c r="D22" s="38" t="s">
         <v>282</v>
       </c>
-      <c r="E22" s="35" t="s">
+      <c r="E22" s="39" t="s">
         <v>283</v>
       </c>
-      <c r="F22" s="36" t="s">
+      <c r="F22" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="37" t="s">
+      <c r="A23" s="41" t="s">
         <v>145</v>
       </c>
-      <c r="B23" s="42" t="s">
+      <c r="B23" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="C23" s="38" t="s">
+      <c r="C23" s="42" t="s">
         <v>276</v>
       </c>
-      <c r="D23" s="38" t="s">
+      <c r="D23" s="42" t="s">
         <v>148</v>
       </c>
-      <c r="E23" s="39" t="s">
+      <c r="E23" s="43" t="s">
         <v>278</v>
       </c>
-      <c r="F23" s="40" t="s">
+      <c r="F23" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="32" t="s">
+      <c r="A24" s="36" t="s">
         <v>152</v>
       </c>
-      <c r="B24" s="42" t="s">
+      <c r="B24" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="C24" s="34" t="s">
+      <c r="C24" s="38" t="s">
         <v>276</v>
       </c>
-      <c r="D24" s="34" t="s">
+      <c r="D24" s="38" t="s">
         <v>154</v>
       </c>
-      <c r="E24" s="35" t="s">
+      <c r="E24" s="39" t="s">
         <v>278</v>
       </c>
-      <c r="F24" s="36" t="s">
+      <c r="F24" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="37" t="s">
+      <c r="A25" s="41" t="s">
         <v>157</v>
       </c>
-      <c r="B25" s="42" t="s">
+      <c r="B25" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="C25" s="38" t="s">
+      <c r="C25" s="42" t="s">
         <v>276</v>
       </c>
-      <c r="D25" s="38" t="s">
+      <c r="D25" s="42" t="s">
         <v>159</v>
       </c>
-      <c r="E25" s="39" t="s">
+      <c r="E25" s="43" t="s">
         <v>281</v>
       </c>
-      <c r="F25" s="40" t="s">
+      <c r="F25" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="32" t="s">
+      <c r="A26" s="36" t="s">
         <v>163</v>
       </c>
-      <c r="B26" s="42" t="s">
+      <c r="B26" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="C26" s="34" t="s">
+      <c r="C26" s="38" t="s">
         <v>276</v>
       </c>
-      <c r="D26" s="34" t="s">
+      <c r="D26" s="38" t="s">
         <v>165</v>
       </c>
-      <c r="E26" s="35" t="s">
+      <c r="E26" s="39" t="s">
         <v>281</v>
       </c>
-      <c r="F26" s="36" t="s">
+      <c r="F26" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="37" t="s">
+      <c r="A27" s="41" t="s">
         <v>170</v>
       </c>
-      <c r="B27" s="43" t="s">
+      <c r="B27" s="47" t="s">
         <v>171</v>
       </c>
-      <c r="C27" s="38" t="s">
+      <c r="C27" s="42" t="s">
         <v>284</v>
       </c>
-      <c r="D27" s="38" t="s">
+      <c r="D27" s="42" t="s">
         <v>285</v>
       </c>
-      <c r="E27" s="39" t="s">
+      <c r="E27" s="43" t="s">
         <v>286</v>
       </c>
-      <c r="F27" s="40" t="s">
+      <c r="F27" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="32" t="s">
+      <c r="A28" s="36" t="s">
         <v>179</v>
       </c>
-      <c r="B28" s="43" t="s">
+      <c r="B28" s="47" t="s">
         <v>171</v>
       </c>
-      <c r="C28" s="34" t="s">
+      <c r="C28" s="38" t="s">
         <v>284</v>
       </c>
-      <c r="D28" s="34" t="s">
+      <c r="D28" s="38" t="s">
         <v>287</v>
       </c>
-      <c r="E28" s="35" t="s">
+      <c r="E28" s="39" t="s">
         <v>286</v>
       </c>
-      <c r="F28" s="36" t="s">
+      <c r="F28" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="37" t="s">
+      <c r="A29" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="B29" s="43" t="s">
+      <c r="B29" s="47" t="s">
         <v>171</v>
       </c>
-      <c r="C29" s="38" t="s">
+      <c r="C29" s="42" t="s">
         <v>284</v>
       </c>
-      <c r="D29" s="38" t="s">
+      <c r="D29" s="42" t="s">
         <v>288</v>
       </c>
-      <c r="E29" s="39" t="s">
+      <c r="E29" s="43" t="s">
         <v>286</v>
       </c>
-      <c r="F29" s="40" t="s">
+      <c r="F29" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="32" t="s">
+      <c r="A30" s="36" t="s">
         <v>189</v>
       </c>
-      <c r="B30" s="43" t="s">
+      <c r="B30" s="47" t="s">
         <v>171</v>
       </c>
-      <c r="C30" s="34" t="s">
+      <c r="C30" s="38" t="s">
         <v>284</v>
       </c>
-      <c r="D30" s="34" t="s">
+      <c r="D30" s="38" t="s">
         <v>289</v>
       </c>
-      <c r="E30" s="35" t="s">
+      <c r="E30" s="39" t="s">
         <v>286</v>
       </c>
-      <c r="F30" s="36" t="s">
+      <c r="F30" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="37" t="s">
+      <c r="A31" s="41" t="s">
         <v>195</v>
       </c>
-      <c r="B31" s="43" t="s">
+      <c r="B31" s="47" t="s">
         <v>171</v>
       </c>
-      <c r="C31" s="38" t="s">
+      <c r="C31" s="42" t="s">
         <v>284</v>
       </c>
-      <c r="D31" s="38" t="s">
+      <c r="D31" s="42" t="s">
         <v>197</v>
       </c>
-      <c r="E31" s="39" t="s">
+      <c r="E31" s="43" t="s">
         <v>290</v>
       </c>
-      <c r="F31" s="40" t="s">
+      <c r="F31" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="32" t="s">
+      <c r="A32" s="36" t="s">
         <v>201</v>
       </c>
-      <c r="B32" s="44" t="s">
+      <c r="B32" s="48" t="s">
         <v>202</v>
       </c>
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="38" t="s">
         <v>291</v>
       </c>
-      <c r="D32" s="34" t="s">
+      <c r="D32" s="38" t="s">
         <v>204</v>
       </c>
-      <c r="E32" s="35" t="s">
+      <c r="E32" s="39" t="s">
         <v>292</v>
       </c>
-      <c r="F32" s="36" t="s">
+      <c r="F32" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="37" t="s">
+      <c r="A33" s="41" t="s">
         <v>208</v>
       </c>
-      <c r="B33" s="44" t="s">
+      <c r="B33" s="48" t="s">
         <v>202</v>
       </c>
-      <c r="C33" s="38" t="s">
+      <c r="C33" s="42" t="s">
         <v>291</v>
       </c>
-      <c r="D33" s="38" t="s">
+      <c r="D33" s="42" t="s">
         <v>209</v>
       </c>
-      <c r="E33" s="39" t="s">
+      <c r="E33" s="43" t="s">
         <v>292</v>
       </c>
-      <c r="F33" s="40" t="s">
+      <c r="F33" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="32" t="s">
+      <c r="A34" s="36" t="s">
         <v>211</v>
       </c>
-      <c r="B34" s="44" t="s">
+      <c r="B34" s="48" t="s">
         <v>202</v>
       </c>
-      <c r="C34" s="34" t="s">
+      <c r="C34" s="38" t="s">
         <v>291</v>
       </c>
-      <c r="D34" s="34" t="s">
+      <c r="D34" s="38" t="s">
         <v>213</v>
       </c>
-      <c r="E34" s="35" t="s">
+      <c r="E34" s="39" t="s">
         <v>292</v>
       </c>
-      <c r="F34" s="36" t="s">
+      <c r="F34" s="40" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="37" t="s">
+      <c r="A35" s="41" t="s">
         <v>217</v>
       </c>
-      <c r="B35" s="44" t="s">
+      <c r="B35" s="48" t="s">
         <v>202</v>
       </c>
-      <c r="C35" s="38" t="s">
+      <c r="C35" s="42" t="s">
         <v>291</v>
       </c>
-      <c r="D35" s="38" t="s">
+      <c r="D35" s="42" t="s">
         <v>218</v>
       </c>
-      <c r="E35" s="39" t="s">
+      <c r="E35" s="43" t="s">
         <v>292</v>
       </c>
-      <c r="F35" s="40" t="s">
+      <c r="F35" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="32" t="s">
+      <c r="A36" s="36" t="s">
         <v>222</v>
       </c>
-      <c r="B36" s="44" t="s">
+      <c r="B36" s="48" t="s">
         <v>202</v>
       </c>
-      <c r="C36" s="34" t="s">
+      <c r="C36" s="38" t="s">
         <v>291</v>
       </c>
-      <c r="D36" s="34" t="s">
+      <c r="D36" s="38" t="s">
         <v>223</v>
       </c>
-      <c r="E36" s="35" t="s">
+      <c r="E36" s="39" t="s">
         <v>292</v>
       </c>
-      <c r="F36" s="36" t="s">
+      <c r="F36" s="40" t="s">
         <v>260</v>
       </c>
     </row>
@@ -4891,225 +4922,225 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="22" t="s">
         <v>293</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
     </row>
     <row r="3" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="23" t="s">
         <v>294</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="49" t="s">
         <v>295</v>
       </c>
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="49" t="s">
         <v>229</v>
       </c>
-      <c r="C4" s="45" t="s">
+      <c r="C4" s="49" t="s">
         <v>296</v>
       </c>
-      <c r="D4" s="45" t="s">
+      <c r="D4" s="49" t="s">
         <v>297</v>
       </c>
-      <c r="E4" s="45" t="s">
+      <c r="E4" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="F4" s="45" t="s">
+      <c r="F4" s="49" t="s">
         <v>299</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="46" t="n">
+      <c r="A5" s="50" t="n">
         <f aca="false">COUNTIF('Test Cases'!A5:A41,"TC-*")</f>
         <v>33</v>
       </c>
-      <c r="B5" s="47" t="n">
+      <c r="B5" s="51" t="n">
         <f aca="false">COUNTIF('Test Cases'!A5:A41,"TC-*")</f>
         <v>33</v>
       </c>
-      <c r="C5" s="46" t="s">
+      <c r="C5" s="50" t="s">
         <v>246</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="50" t="s">
         <v>248</v>
       </c>
-      <c r="E5" s="46" t="n">
-        <f aca="false">COUNTIF('Test Cases'!B5:B41,"Y")</f>
+      <c r="E5" s="50" t="n">
+        <f aca="false">COUNTIF('Test Cases'!B5:B41,"✓")</f>
         <v>4</v>
       </c>
-      <c r="F5" s="46" t="n">
-        <f aca="false">COUNTIF('Test Cases'!D5:D41,"Y")</f>
+      <c r="F5" s="50" t="n">
+        <f aca="false">COUNTIF('Test Cases'!D5:D41,"✓")</f>
         <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="23" t="s">
         <v>300</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="24" t="s">
         <v>235</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="24" t="s">
         <v>301</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="24" t="s">
         <v>235</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="24" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Functional")</f>
         <v>6</v>
       </c>
-      <c r="C9" s="22" t="str">
+      <c r="C9" s="26" t="str">
         <f aca="false">TEXT(B9/COUNTIF('Test Cases'!A5:A41,"TC-*"),"0%")</f>
         <v>18%</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="E9" s="22" t="n">
+      <c r="E9" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Access Control")</f>
         <v>5</v>
       </c>
-      <c r="F9" s="22" t="str">
+      <c r="F9" s="26" t="str">
         <f aca="false">TEXT(E9/COUNTIF('Test Cases'!A5:A41,"TC-*"),"0%")</f>
         <v>15%</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24" t="s">
+      <c r="A10" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Boundary")</f>
         <v>8</v>
       </c>
-      <c r="C10" s="22" t="str">
+      <c r="C10" s="26" t="str">
         <f aca="false">TEXT(B10/COUNTIF('Test Cases'!A5:A41,"TC-*"),"0%")</f>
         <v>24%</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="31" t="s">
         <v>202</v>
       </c>
-      <c r="E10" s="22" t="n">
+      <c r="E10" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Performance")</f>
         <v>5</v>
       </c>
-      <c r="F10" s="22" t="str">
+      <c r="F10" s="26" t="str">
         <f aca="false">TEXT(E10/COUNTIF('Test Cases'!A5:A41,"TC-*"),"0%")</f>
         <v>15%</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="29" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B11" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!F5:F41,"Security")</f>
         <v>9</v>
       </c>
-      <c r="C11" s="22" t="str">
+      <c r="C11" s="26" t="str">
         <f aca="false">TEXT(B11/COUNTIF('Test Cases'!A5:A41,"TC-*"),"0%")</f>
         <v>27%</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="23" t="s">
         <v>302</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="24" t="s">
         <v>235</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="24" t="s">
         <v>303</v>
       </c>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="48" t="s">
+      <c r="A15" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="22" t="n">
+      <c r="B15" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!O5:O41,"Pass")</f>
         <v>32</v>
       </c>
-      <c r="C15" s="49" t="s">
+      <c r="C15" s="53" t="s">
         <v>304</v>
       </c>
-      <c r="D15" s="49"/>
-      <c r="E15" s="49"/>
-      <c r="F15" s="49"/>
+      <c r="D15" s="53"/>
+      <c r="E15" s="53"/>
+      <c r="F15" s="53"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="50" t="s">
+      <c r="A16" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="B16" s="22" t="n">
+      <c r="B16" s="26" t="n">
         <f aca="false">COUNTIF('Test Cases'!O5:O41,"Observation")</f>
         <v>1</v>
       </c>
-      <c r="C16" s="49" t="s">
+      <c r="C16" s="53" t="s">
         <v>305</v>
       </c>
-      <c r="D16" s="49"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="49"/>
+      <c r="D16" s="53"/>
+      <c r="E16" s="53"/>
+      <c r="F16" s="53"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="32" t="s">
         <v>306</v>
       </c>
-      <c r="B17" s="51" t="s">
+      <c r="B17" s="55" t="s">
         <v>307</v>
       </c>
-      <c r="C17" s="51"/>
-      <c r="D17" s="51"/>
-      <c r="E17" s="51"/>
-      <c r="F17" s="51"/>
+      <c r="C17" s="55"/>
+      <c r="D17" s="55"/>
+      <c r="E17" s="55"/>
+      <c r="F17" s="55"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -5144,244 +5175,244 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="22" t="s">
         <v>308</v>
       </c>
-      <c r="B1" s="18"/>
+      <c r="B1" s="22"/>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="56" t="s">
         <v>309</v>
       </c>
-      <c r="B2" s="52"/>
+      <c r="B2" s="56"/>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="57" t="s">
         <v>310</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="58" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="57" t="s">
         <v>312</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="58" t="s">
         <v>313</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="53" t="s">
+      <c r="A5" s="57" t="s">
         <v>314</v>
       </c>
-      <c r="B5" s="54" t="s">
+      <c r="B5" s="58" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="53" t="s">
+      <c r="A6" s="57" t="s">
         <v>316</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="58" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="53" t="s">
+      <c r="A7" s="57" t="s">
         <v>318</v>
       </c>
-      <c r="B7" s="54" t="s">
+      <c r="B7" s="58" t="s">
         <v>319</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="52" t="s">
+      <c r="A8" s="56" t="s">
         <v>320</v>
       </c>
-      <c r="B8" s="52"/>
+      <c r="B8" s="56"/>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="53" t="s">
+      <c r="A9" s="57" t="s">
         <v>321</v>
       </c>
-      <c r="B9" s="54" t="s">
+      <c r="B9" s="58" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="53" t="s">
+      <c r="A10" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="54" t="s">
+      <c r="B10" s="58" t="s">
         <v>323</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="53" t="s">
+      <c r="A11" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="54" t="s">
+      <c r="B11" s="58" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="53" t="s">
+      <c r="A12" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="54" t="s">
+      <c r="B12" s="58" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="53" t="s">
+      <c r="A13" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="54" t="s">
+      <c r="B13" s="58" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="53" t="s">
+      <c r="A14" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="54" t="s">
+      <c r="B14" s="58" t="s">
         <v>327</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="52" t="s">
+      <c r="A15" s="56" t="s">
         <v>328</v>
       </c>
-      <c r="B15" s="52"/>
+      <c r="B15" s="56"/>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="55" t="s">
+      <c r="A16" s="59" t="s">
         <v>329</v>
       </c>
-      <c r="B16" s="54" t="s">
+      <c r="B16" s="58" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="56" t="s">
+      <c r="A17" s="60" t="s">
         <v>330</v>
       </c>
-      <c r="B17" s="54" t="s">
+      <c r="B17" s="58" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="57" t="s">
+      <c r="A18" s="61" t="s">
         <v>332</v>
       </c>
-      <c r="B18" s="54" t="s">
+      <c r="B18" s="58" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="58" t="s">
+      <c r="A19" s="62" t="s">
         <v>334</v>
       </c>
-      <c r="B19" s="54" t="s">
+      <c r="B19" s="58" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="59" t="s">
+      <c r="A20" s="63" t="s">
         <v>335</v>
       </c>
-      <c r="B20" s="54" t="s">
+      <c r="B20" s="58" t="s">
         <v>336</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="52" t="s">
+      <c r="A21" s="56" t="s">
         <v>337</v>
       </c>
-      <c r="B21" s="52"/>
+      <c r="B21" s="56"/>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="53" t="s">
+      <c r="A22" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="54" t="s">
+      <c r="B22" s="58" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="53" t="s">
+      <c r="A23" s="57" t="s">
         <v>70</v>
       </c>
-      <c r="B23" s="54" t="s">
+      <c r="B23" s="58" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="53" t="s">
+      <c r="A24" s="57" t="s">
         <v>117</v>
       </c>
-      <c r="B24" s="54" t="s">
+      <c r="B24" s="58" t="s">
         <v>340</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="53" t="s">
+      <c r="A25" s="57" t="s">
         <v>171</v>
       </c>
-      <c r="B25" s="54" t="s">
+      <c r="B25" s="58" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="53" t="s">
+      <c r="A26" s="57" t="s">
         <v>202</v>
       </c>
-      <c r="B26" s="54" t="s">
+      <c r="B26" s="58" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="52" t="s">
+      <c r="A27" s="56" t="s">
         <v>343</v>
       </c>
-      <c r="B27" s="52"/>
+      <c r="B27" s="56"/>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="53" t="s">
+      <c r="A28" s="57" t="s">
         <v>344</v>
       </c>
-      <c r="B28" s="54" t="s">
+      <c r="B28" s="58" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="53" t="s">
+      <c r="A29" s="57" t="s">
         <v>346</v>
       </c>
-      <c r="B29" s="54" t="s">
+      <c r="B29" s="58" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="53" t="s">
+      <c r="A30" s="57" t="s">
         <v>348</v>
       </c>
-      <c r="B30" s="54" t="s">
+      <c r="B30" s="58" t="s">
         <v>349</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="52" t="s">
+      <c r="A31" s="56" t="s">
         <v>350</v>
       </c>
-      <c r="B31" s="52"/>
+      <c r="B31" s="56"/>
     </row>
     <row r="32" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="53" t="s">
+      <c r="A32" s="57" t="s">
         <v>351</v>
       </c>
-      <c r="B32" s="54" t="s">
+      <c r="B32" s="58" t="s">
         <v>352</v>
       </c>
     </row>

</xml_diff>